<commit_message>
Primera prueba adición de sorteo estocastico
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -1004,14 +1004,14 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[2, 6, 8, 2]</t>
+          <t>[2, 6, 2]</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>2486</v>
+        <v>1519</v>
       </c>
       <c r="J4" t="n">
-        <v>72.44731374037281</v>
+        <v>72.36542765017174</v>
       </c>
       <c r="K4" t="b">
         <v>1</v>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="AO4" t="n">
-        <v>11.40413399857448</v>
+        <v>45.86600142551675</v>
       </c>
       <c r="AP4" t="n">
         <v>0</v>
@@ -2368,7 +2368,7 @@
         <v>561.4</v>
       </c>
       <c r="J2" t="n">
-        <v>1031.922685146332</v>
+        <v>1117.89514875412</v>
       </c>
       <c r="K2" t="n">
         <v>0.1387406616862326</v>

</xml_diff>

<commit_message>
Primera prueba adición MIP dinamico
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS11"/>
+  <dimension ref="A1:BA11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -532,127 +532,167 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>Oracle Status</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>Oracle Route</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>Oracle Reward</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Oracle Duration</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Oracle Valid</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>2Opt Route</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>2Opt Reward</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>2Opt Duration</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>2Opt Valid</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>GA Status</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>GA Route</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>GA Reward</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>GA Duration</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>GA Valid</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>LNS Status</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>LNS Route</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>LNS Reward</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>LNS Duration</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>LNS Valid</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Status</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Route</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Reward</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Duration</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Valid</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>DRL Gap (%)</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Gap (%)</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>2Opt Gap (%)</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>GA Gap (%)</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>LNS Gap (%)</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Gap (%)</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>Oracle Gap vs DRL Real (%)</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>Oracle Gap vs RH-Greedy (%)</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>Oracle Gap vs MIP Static (%)</t>
         </is>
       </c>
     </row>
@@ -729,22 +769,22 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>[0, 1, 6, 0]</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>1964</v>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>[0, 6, 1, 0]</t>
+        </is>
       </c>
       <c r="W2" t="n">
+        <v>2041</v>
+      </c>
+      <c r="X2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="X2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+      <c r="Y2" t="b">
+        <v>1</v>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
@@ -767,54 +807,82 @@
       </c>
       <c r="AE2" t="inlineStr">
         <is>
+          <t>[0, 1, 6, 0]</t>
+        </is>
+      </c>
+      <c r="AF2" t="n">
+        <v>1964</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AH2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ2" t="inlineStr">
+        <is>
           <t>[0, 6, 0]</t>
         </is>
       </c>
-      <c r="AF2" t="n">
+      <c r="AK2" t="n">
         <v>1735</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AL2" t="n">
         <v>55.44764714720212</v>
       </c>
-      <c r="AH2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AM2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="AK2" t="n">
+      <c r="AP2" t="n">
         <v>1964</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AQ2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AM2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO2" t="n">
+      <c r="AR2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
         <v>-3.920570264765784</v>
       </c>
-      <c r="AP2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR2" t="n">
+      <c r="AU2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW2" t="n">
         <v>11.65987780040733</v>
       </c>
-      <c r="AS2" t="n">
-        <v>0</v>
+      <c r="AX2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
+        <v>10.43606075453209</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>3.77266046055855</v>
       </c>
     </row>
     <row r="3">
@@ -890,92 +958,120 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>[1, 0, 6, 1]</t>
+        </is>
+      </c>
+      <c r="W3" t="n">
+        <v>1635</v>
+      </c>
+      <c r="X3" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="Y3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
           <t>[1, 8, 2, 1]</t>
         </is>
       </c>
-      <c r="V3" t="n">
+      <c r="AA3" t="n">
         <v>-669</v>
       </c>
-      <c r="W3" t="n">
+      <c r="AB3" t="n">
         <v>69.40771788690013</v>
       </c>
-      <c r="X3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AC3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="AA3" t="n">
+      <c r="AF3" t="n">
         <v>1571</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AG3" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AC3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AH3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>[1, 2, 8, 1]</t>
         </is>
       </c>
-      <c r="AF3" t="n">
+      <c r="AK3" t="n">
         <v>-773</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AL3" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="AH3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr">
+      <c r="AM3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="AK3" t="n">
+      <c r="AP3" t="n">
         <v>1571</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="AQ3" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AM3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO3" t="n">
+      <c r="AR3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
         <v>-5.410566518141311</v>
       </c>
-      <c r="AP3" t="n">
+      <c r="AU3" t="n">
         <v>142.5843411839593</v>
       </c>
-      <c r="AQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR3" t="n">
+      <c r="AV3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW3" t="n">
         <v>149.2043284532145</v>
       </c>
-      <c r="AS3" t="n">
-        <v>0</v>
+      <c r="AX3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY3" t="n">
+        <v>-1.284403669724771</v>
+      </c>
+      <c r="AZ3" t="n">
+        <v>28.80733944954128</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>3.914373088685015</v>
       </c>
     </row>
     <row r="4">
@@ -1051,22 +1147,22 @@
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>[2, 8, 6, 2]</t>
-        </is>
-      </c>
-      <c r="V4" t="n">
-        <v>2806</v>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>[2, 1, 8, 2]</t>
+        </is>
       </c>
       <c r="W4" t="n">
-        <v>72.44731374037281</v>
-      </c>
-      <c r="X4" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+        <v>1807</v>
+      </c>
+      <c r="X4" t="n">
+        <v>70.15987690240343</v>
+      </c>
+      <c r="Y4" t="b">
+        <v>1</v>
       </c>
       <c r="Z4" t="inlineStr">
         <is>
@@ -1089,54 +1185,82 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
+          <t>[2, 8, 6, 2]</t>
+        </is>
+      </c>
+      <c r="AF4" t="n">
+        <v>2806</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>72.44731374037281</v>
+      </c>
+      <c r="AH4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="AF4" t="n">
+      <c r="AK4" t="n">
         <v>976</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AL4" t="n">
         <v>72.45471862628276</v>
       </c>
-      <c r="AH4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
+      <c r="AM4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="AK4" t="n">
+      <c r="AP4" t="n">
         <v>2806</v>
       </c>
-      <c r="AL4" t="n">
+      <c r="AQ4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AM4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AN4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO4" t="n">
+      <c r="AR4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="n">
         <v>45.86600142551675</v>
       </c>
-      <c r="AP4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR4" t="n">
+      <c r="AU4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW4" t="n">
         <v>65.21739130434783</v>
       </c>
-      <c r="AS4" t="n">
-        <v>0</v>
+      <c r="AX4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY4" t="n">
+        <v>15.93801881571666</v>
+      </c>
+      <c r="AZ4" t="n">
+        <v>167.5705589374654</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>-55.28500276701715</v>
       </c>
     </row>
     <row r="5">
@@ -1212,22 +1336,22 @@
       </c>
       <c r="U5" t="inlineStr">
         <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="V5" t="n">
-        <v>1281</v>
-      </c>
       <c r="W5" t="n">
+        <v>1344</v>
+      </c>
+      <c r="X5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="X5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+      <c r="Y5" t="b">
+        <v>1</v>
       </c>
       <c r="Z5" t="inlineStr">
         <is>
@@ -1281,23 +1405,51 @@
       <c r="AM5" t="b">
         <v>1</v>
       </c>
-      <c r="AN5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO5" t="n">
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO5" t="inlineStr">
+        <is>
+          <t>[3, 4, 3]</t>
+        </is>
+      </c>
+      <c r="AP5" t="n">
+        <v>1281</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="AR5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
         <v>-4.918032786885246</v>
       </c>
-      <c r="AP5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS5" t="n">
-        <v>0</v>
+      <c r="AU5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ5" t="n">
+        <v>4.613095238095238</v>
+      </c>
+      <c r="BA5" t="n">
+        <v>4.6875</v>
       </c>
     </row>
     <row r="6">
@@ -1373,22 +1525,22 @@
       </c>
       <c r="U6" t="inlineStr">
         <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="V6" t="n">
-        <v>1080</v>
-      </c>
       <c r="W6" t="n">
+        <v>1281</v>
+      </c>
+      <c r="X6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="X6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+      <c r="Y6" t="b">
+        <v>1</v>
       </c>
       <c r="Z6" t="inlineStr">
         <is>
@@ -1442,23 +1594,51 @@
       <c r="AM6" t="b">
         <v>1</v>
       </c>
-      <c r="AN6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO6" t="n">
+      <c r="AN6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO6" t="inlineStr">
+        <is>
+          <t>[4, 3, 4]</t>
+        </is>
+      </c>
+      <c r="AP6" t="n">
+        <v>1080</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="AR6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
         <v>-18.61111111111111</v>
       </c>
-      <c r="AP6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS6" t="n">
-        <v>0</v>
+      <c r="AU6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ6" t="n">
+        <v>15.69086651053864</v>
+      </c>
+      <c r="BA6" t="n">
+        <v>15.69086651053864</v>
       </c>
     </row>
     <row r="7">
@@ -1534,22 +1714,22 @@
       </c>
       <c r="U7" t="inlineStr">
         <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="V7" t="n">
-        <v>774</v>
-      </c>
       <c r="W7" t="n">
+        <v>781</v>
+      </c>
+      <c r="X7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="X7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+      <c r="Y7" t="b">
+        <v>1</v>
       </c>
       <c r="Z7" t="inlineStr">
         <is>
@@ -1603,23 +1783,51 @@
       <c r="AM7" t="b">
         <v>1</v>
       </c>
-      <c r="AN7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO7" t="n">
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>[5, 3, 5]</t>
+        </is>
+      </c>
+      <c r="AP7" t="n">
+        <v>774</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>48.69171070169158</v>
+      </c>
+      <c r="AR7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="n">
         <v>-0.9043927648578811</v>
       </c>
-      <c r="AP7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>0</v>
+      <c r="AU7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ7" t="n">
+        <v>0.8962868117797695</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0.8962868117797695</v>
       </c>
     </row>
     <row r="8">
@@ -1695,22 +1903,22 @@
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>[6, 0, 1, 6]</t>
-        </is>
-      </c>
-      <c r="V8" t="n">
-        <v>1964</v>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>[6, 1, 0, 6]</t>
+        </is>
       </c>
       <c r="W8" t="n">
+        <v>2032</v>
+      </c>
+      <c r="X8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="X8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+      <c r="Y8" t="b">
+        <v>1</v>
       </c>
       <c r="Z8" t="inlineStr">
         <is>
@@ -1764,23 +1972,51 @@
       <c r="AM8" t="b">
         <v>1</v>
       </c>
-      <c r="AN8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO8" t="n">
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>[6, 0, 1, 6]</t>
+        </is>
+      </c>
+      <c r="AP8" t="n">
+        <v>1964</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AR8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
         <v>-2.90224032586558</v>
       </c>
-      <c r="AP8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>0</v>
+      <c r="AU8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY8" t="n">
+        <v>0.5413385826771654</v>
+      </c>
+      <c r="AZ8" t="n">
+        <v>7.97244094488189</v>
+      </c>
+      <c r="BA8" t="n">
+        <v>3.346456692913386</v>
       </c>
     </row>
     <row r="9">
@@ -1856,22 +2092,22 @@
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>[7, 8, 6, 7]</t>
-        </is>
-      </c>
-      <c r="V9" t="n">
-        <v>2634</v>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>[7, 6, 8, 7]</t>
+        </is>
       </c>
       <c r="W9" t="n">
+        <v>2169</v>
+      </c>
+      <c r="X9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="X9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+      <c r="Y9" t="b">
+        <v>1</v>
       </c>
       <c r="Z9" t="inlineStr">
         <is>
@@ -1925,23 +2161,51 @@
       <c r="AM9" t="b">
         <v>1</v>
       </c>
-      <c r="AN9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO9" t="n">
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>[7, 8, 6, 7]</t>
+        </is>
+      </c>
+      <c r="AP9" t="n">
+        <v>2634</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>76.25197526044872</v>
+      </c>
+      <c r="AR9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT9" t="n">
         <v>18.00286327845383</v>
       </c>
-      <c r="AP9" t="n">
+      <c r="AU9" t="n">
         <v>5.72655690765927</v>
       </c>
-      <c r="AQ9" t="n">
+      <c r="AV9" t="n">
         <v>5.72655690765927</v>
       </c>
-      <c r="AR9" t="n">
+      <c r="AW9" t="n">
         <v>5.72655690765927</v>
       </c>
-      <c r="AS9" t="n">
+      <c r="AX9" t="n">
         <v>5.72655690765927</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>-5.624711848778239</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>36.42231443061318</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>-28.81512217611802</v>
       </c>
     </row>
     <row r="10">
@@ -2017,22 +2281,22 @@
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>[8, 1, 2, 8]</t>
-        </is>
-      </c>
-      <c r="V10" t="n">
-        <v>1874</v>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>[8, 2, 1, 8]</t>
+        </is>
       </c>
       <c r="W10" t="n">
+        <v>1950</v>
+      </c>
+      <c r="X10" t="n">
         <v>70.15987690240343</v>
       </c>
-      <c r="X10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+      <c r="Y10" t="b">
+        <v>1</v>
       </c>
       <c r="Z10" t="inlineStr">
         <is>
@@ -2086,23 +2350,51 @@
       <c r="AM10" t="b">
         <v>1</v>
       </c>
-      <c r="AN10" t="n">
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>[8, 1, 2, 8]</t>
+        </is>
+      </c>
+      <c r="AP10" t="n">
+        <v>1874</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>70.15987690240343</v>
+      </c>
+      <c r="AR10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AS10" t="n">
         <v>1.387406616862326</v>
       </c>
-      <c r="AO10" t="n">
+      <c r="AT10" t="n">
         <v>8.911419423692637</v>
       </c>
-      <c r="AP10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS10" t="n">
-        <v>0</v>
+      <c r="AU10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY10" t="n">
+        <v>12.46153846153846</v>
+      </c>
+      <c r="AZ10" t="n">
+        <v>23.07692307692308</v>
+      </c>
+      <c r="BA10" t="n">
+        <v>3.897435897435898</v>
       </c>
     </row>
     <row r="11">
@@ -2178,22 +2470,22 @@
       </c>
       <c r="U11" t="inlineStr">
         <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="V11" t="n">
-        <v>-4042</v>
-      </c>
       <c r="W11" t="n">
+        <v>-2000000000</v>
+      </c>
+      <c r="X11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="X11" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
+      <c r="Y11" t="b">
+        <v>1</v>
       </c>
       <c r="Z11" t="inlineStr">
         <is>
@@ -2247,23 +2539,51 @@
       <c r="AM11" t="b">
         <v>1</v>
       </c>
-      <c r="AN11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>0</v>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>[9, 2, 9]</t>
+        </is>
       </c>
       <c r="AP11" t="n">
-        <v>0</v>
+        <v>-4042</v>
       </c>
       <c r="AQ11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR11" t="n">
-        <v>0</v>
+        <v>64.70237352474922</v>
+      </c>
+      <c r="AR11" t="b">
+        <v>1</v>
       </c>
       <c r="AS11" t="n">
         <v>0</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY11" t="n">
+        <v>-99.9997979</v>
+      </c>
+      <c r="AZ11" t="n">
+        <v>-99.9997979</v>
+      </c>
+      <c r="BA11" t="n">
+        <v>-99.9997979</v>
       </c>
     </row>
   </sheetData>
@@ -2368,7 +2688,7 @@
         <v>561.4</v>
       </c>
       <c r="J2" t="n">
-        <v>1117.89514875412</v>
+        <v>1118.594800233841</v>
       </c>
       <c r="K2" t="n">
         <v>0.1387406616862326</v>

</xml_diff>

<commit_message>
Segunda prueba adición MIP dinamico
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="W3" t="n">
-        <v>1635</v>
+        <v>1644</v>
       </c>
       <c r="X3" t="n">
         <v>76.7052345103569</v>
@@ -1065,13 +1065,13 @@
         <v>0</v>
       </c>
       <c r="AY3" t="n">
-        <v>-1.284403669724771</v>
+        <v>-0.7299270072992701</v>
       </c>
       <c r="AZ3" t="n">
-        <v>28.80733944954128</v>
+        <v>29.1970802919708</v>
       </c>
       <c r="BA3" t="n">
-        <v>3.914373088685015</v>
+        <v>4.440389294403893</v>
       </c>
     </row>
     <row r="4">
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="W4" t="n">
-        <v>1807</v>
+        <v>1366</v>
       </c>
       <c r="X4" t="n">
         <v>70.15987690240343</v>
@@ -1254,13 +1254,13 @@
         <v>0</v>
       </c>
       <c r="AY4" t="n">
-        <v>15.93801881571666</v>
+        <v>-11.20058565153734</v>
       </c>
       <c r="AZ4" t="n">
-        <v>167.5705589374654</v>
+        <v>189.385065885798</v>
       </c>
       <c r="BA4" t="n">
-        <v>-55.28500276701715</v>
+        <v>-105.4172767203514</v>
       </c>
     </row>
     <row r="5">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="W8" t="n">
-        <v>2032</v>
+        <v>2021</v>
       </c>
       <c r="X8" t="n">
         <v>76.7052345103569</v>
@@ -2010,13 +2010,13 @@
         <v>0</v>
       </c>
       <c r="AY8" t="n">
-        <v>0.5413385826771654</v>
+        <v>0</v>
       </c>
       <c r="AZ8" t="n">
-        <v>7.97244094488189</v>
+        <v>7.471548738248392</v>
       </c>
       <c r="BA8" t="n">
-        <v>3.346456692913386</v>
+        <v>2.820385947550717</v>
       </c>
     </row>
     <row r="9">
@@ -2097,14 +2097,14 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>[7, 6, 8, 7]</t>
+          <t>[7, 8, 7]</t>
         </is>
       </c>
       <c r="W9" t="n">
-        <v>2169</v>
+        <v>2291</v>
       </c>
       <c r="X9" t="n">
-        <v>76.25197526044872</v>
+        <v>72.81063071208843</v>
       </c>
       <c r="Y9" t="b">
         <v>1</v>
@@ -2199,13 +2199,13 @@
         <v>5.72655690765927</v>
       </c>
       <c r="AY9" t="n">
-        <v>-5.624711848778239</v>
+        <v>0</v>
       </c>
       <c r="AZ9" t="n">
-        <v>36.42231443061318</v>
+        <v>39.80794412920122</v>
       </c>
       <c r="BA9" t="n">
-        <v>-28.81512217611802</v>
+        <v>-21.95547795722392</v>
       </c>
     </row>
     <row r="10">
@@ -2290,10 +2290,10 @@
         </is>
       </c>
       <c r="W10" t="n">
-        <v>1950</v>
+        <v>1707</v>
       </c>
       <c r="X10" t="n">
-        <v>70.15987690240343</v>
+        <v>70.15987690240341</v>
       </c>
       <c r="Y10" t="b">
         <v>1</v>
@@ -2388,13 +2388,13 @@
         <v>0</v>
       </c>
       <c r="AY10" t="n">
-        <v>12.46153846153846</v>
+        <v>0</v>
       </c>
       <c r="AZ10" t="n">
-        <v>23.07692307692308</v>
+        <v>12.12653778558875</v>
       </c>
       <c r="BA10" t="n">
-        <v>3.897435897435898</v>
+        <v>-9.78324545987112</v>
       </c>
     </row>
     <row r="11">
@@ -2479,7 +2479,7 @@
         </is>
       </c>
       <c r="W11" t="n">
-        <v>-2000000000</v>
+        <v>-4042</v>
       </c>
       <c r="X11" t="n">
         <v>64.70237352474922</v>
@@ -2577,13 +2577,13 @@
         <v>0</v>
       </c>
       <c r="AY11" t="n">
-        <v>-99.9997979</v>
+        <v>0</v>
       </c>
       <c r="AZ11" t="n">
-        <v>-99.9997979</v>
+        <v>0</v>
       </c>
       <c r="BA11" t="n">
-        <v>-99.9997979</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2597,7 +2597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2613,47 +2613,67 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Oracle Avg Reward</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>MIP Avg Reward</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>DRL Avg Reward</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>DRL Real Avg Reward</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Avg Reward</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>2Opt Avg</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>GA Avg</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>LNS Avg</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>DRL Training Time</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>DRL Avg Gap (%)</t>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Avg Gap vs MIP (%)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Avg Gap vs Oracle (%)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Max Gap vs Oracle (%)</t>
         </is>
       </c>
     </row>
@@ -2667,31 +2687,43 @@
         <v>10</v>
       </c>
       <c r="C2" t="n">
+        <v>1043.4</v>
+      </c>
+      <c r="D2" t="n">
         <v>1206.6</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
+        <v>1059.9</v>
+      </c>
+      <c r="F2" t="n">
         <v>1204</v>
       </c>
-      <c r="E2" t="n">
+      <c r="G2" t="n">
         <v>966.6</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1190.6</v>
-      </c>
-      <c r="G2" t="n">
-        <v>750.3</v>
       </c>
       <c r="H2" t="n">
         <v>1190.6</v>
       </c>
       <c r="I2" t="n">
+        <v>750.3</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1190.6</v>
+      </c>
+      <c r="K2" t="n">
         <v>561.4</v>
       </c>
-      <c r="J2" t="n">
-        <v>1118.594800233841</v>
-      </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
+        <v>1137.798395872116</v>
+      </c>
+      <c r="M2" t="n">
         <v>0.1387406616862326</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-1.193051265883661</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resultados iniciales tras reemplazo de Solvers
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X11"/>
+  <dimension ref="A1:AC11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -467,87 +467,112 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>DRL Det Route</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Reward</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Duration</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Valid</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>RH-Greedy Route</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Reward</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Duration</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Valid</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Status</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Route</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Reward</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Duration</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Valid</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Oracle Status</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Oracle Route</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Oracle Reward</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Oracle Duration</t>
-        </is>
-      </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Oracle Valid</t>
+          <t>MIP-Exact Status</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Oracle Gap vs DRL Real (%)</t>
+          <t>MIP-Exact Route</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Oracle Gap vs RH-Greedy (%)</t>
+          <t>MIP-Exact Reward</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>Oracle Gap vs HGA-LNS (%)</t>
+          <t>MIP-Exact Duration</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>MIP-Exact Valid</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>MIP-Exact Gap vs DRL Det (%)</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>MIP-Exact Gap vs DRL Real (%)</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>MIP-Exact Gap vs RH-Greedy (%)</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>MIP-Exact Gap vs HGA-LNS (%)</t>
         </is>
       </c>
     </row>
@@ -581,7 +606,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>2054</v>
+        <v>2041</v>
       </c>
       <c r="J2" t="n">
         <v>76.7052345103569</v>
@@ -591,49 +616,66 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
+          <t>[0, 6, 1, 0]</t>
+        </is>
+      </c>
+      <c r="M2" t="n">
+        <v>2054</v>
+      </c>
+      <c r="N2" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="O2" t="b">
+        <v>1</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>[0, 1, 6, 0]</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="R2" t="n">
         <v>1727</v>
       </c>
-      <c r="O2" t="n">
+      <c r="S2" t="n">
         <v>77.62623579449122</v>
       </c>
-      <c r="P2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="b">
+        <v>1</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
         <is>
           <t>[0, 6, 1, 0]</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="W2" t="n">
         <v>2041</v>
       </c>
-      <c r="T2" t="n">
+      <c r="X2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="U2" t="b">
-        <v>1</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
+      <c r="Y2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB2" t="n">
         <v>-0.6369426751592357</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AC2" t="n">
         <v>15.38461538461539</v>
       </c>
     </row>
@@ -663,64 +705,81 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>[1, 6, 8, 1]</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>1656</v>
+      </c>
+      <c r="J3" t="n">
+        <v>76.66491525851202</v>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>[1, 2, 8, 1]</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="M3" t="n">
         <v>1164</v>
       </c>
-      <c r="J3" t="n">
+      <c r="N3" t="n">
         <v>69.40771788690012</v>
       </c>
-      <c r="K3" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="b">
+        <v>1</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>[1, 6, 0, 1]</t>
         </is>
       </c>
-      <c r="N3" t="n">
+      <c r="R3" t="n">
         <v>1928</v>
       </c>
-      <c r="O3" t="n">
+      <c r="S3" t="n">
         <v>77.62623579449122</v>
       </c>
-      <c r="P3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>[1, 0, 6, 1]</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
-        <v>1644</v>
-      </c>
-      <c r="T3" t="n">
-        <v>76.7052345103569</v>
-      </c>
-      <c r="U3" t="b">
-        <v>1</v>
-      </c>
-      <c r="V3" t="n">
-        <v>-0.7299270072992701</v>
+      <c r="T3" t="b">
+        <v>1</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>[1, 6, 8, 1]</t>
+        </is>
       </c>
       <c r="W3" t="n">
-        <v>29.1970802919708</v>
+        <v>1656</v>
       </c>
       <c r="X3" t="n">
-        <v>-17.27493917274939</v>
+        <v>76.66491525851202</v>
+      </c>
+      <c r="Y3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>29.71014492753623</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>-16.42512077294686</v>
       </c>
     </row>
     <row r="4">
@@ -753,7 +812,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>-1221</v>
+        <v>2486</v>
       </c>
       <c r="J4" t="n">
         <v>72.44731374037281</v>
@@ -763,50 +822,67 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
+          <t>[2, 6, 8, 2]</t>
+        </is>
+      </c>
+      <c r="M4" t="n">
+        <v>-1221</v>
+      </c>
+      <c r="N4" t="n">
+        <v>72.44731374037281</v>
+      </c>
+      <c r="O4" t="b">
+        <v>1</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>[2, 8, 6, 2]</t>
         </is>
       </c>
-      <c r="N4" t="n">
+      <c r="R4" t="n">
         <v>976</v>
       </c>
-      <c r="O4" t="n">
+      <c r="S4" t="n">
         <v>72.45471862628276</v>
       </c>
-      <c r="P4" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
-        <is>
-          <t>[2, 1, 8, 2]</t>
-        </is>
-      </c>
-      <c r="S4" t="n">
-        <v>1366</v>
-      </c>
-      <c r="T4" t="n">
-        <v>70.15987690240343</v>
-      </c>
-      <c r="U4" t="b">
-        <v>1</v>
-      </c>
-      <c r="V4" t="n">
-        <v>-11.20058565153734</v>
+      <c r="T4" t="b">
+        <v>1</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>[2, 6, 8, 2]</t>
+        </is>
       </c>
       <c r="W4" t="n">
-        <v>189.385065885798</v>
+        <v>2486</v>
       </c>
       <c r="X4" t="n">
-        <v>28.55051244509517</v>
+        <v>72.44731374037281</v>
+      </c>
+      <c r="Y4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>38.89782783588093</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>149.1150442477876</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>60.74014481094127</v>
       </c>
     </row>
     <row r="5">
@@ -839,7 +915,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>1282</v>
+        <v>1344</v>
       </c>
       <c r="J5" t="n">
         <v>40.68356024804761</v>
@@ -849,49 +925,66 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
+      <c r="M5" t="n">
+        <v>1282</v>
+      </c>
       <c r="N5" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="O5" t="b">
+        <v>1</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>[3, 4, 3]</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
         <v>1344</v>
       </c>
-      <c r="O5" t="n">
+      <c r="S5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="P5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q5" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="b">
+        <v>1</v>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="S5" t="n">
+      <c r="W5" t="n">
         <v>1344</v>
       </c>
-      <c r="T5" t="n">
+      <c r="X5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="U5" t="b">
-        <v>1</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" t="n">
+      <c r="Y5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB5" t="n">
         <v>4.613095238095238</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AC5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -925,7 +1018,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>1080</v>
+        <v>1281</v>
       </c>
       <c r="J6" t="n">
         <v>40.68356024804761</v>
@@ -935,49 +1028,66 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
+      <c r="M6" t="n">
+        <v>1080</v>
+      </c>
       <c r="N6" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="O6" t="b">
+        <v>1</v>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>[4, 3, 4]</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
         <v>1281</v>
       </c>
-      <c r="O6" t="n">
+      <c r="S6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="P6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
+      <c r="T6" t="b">
+        <v>1</v>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="S6" t="n">
+      <c r="W6" t="n">
         <v>1281</v>
       </c>
-      <c r="T6" t="n">
+      <c r="X6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="U6" t="b">
-        <v>1</v>
-      </c>
-      <c r="V6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W6" t="n">
+      <c r="Y6" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB6" t="n">
         <v>15.69086651053864</v>
       </c>
-      <c r="X6" t="n">
+      <c r="AC6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1011,7 +1121,7 @@
         </is>
       </c>
       <c r="I7" t="n">
-        <v>774</v>
+        <v>781</v>
       </c>
       <c r="J7" t="n">
         <v>48.69171070169158</v>
@@ -1021,49 +1131,66 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M7" t="inlineStr">
-        <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
+      <c r="M7" t="n">
+        <v>774</v>
+      </c>
       <c r="N7" t="n">
+        <v>48.69171070169158</v>
+      </c>
+      <c r="O7" t="b">
+        <v>1</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>[5, 3, 5]</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
         <v>781</v>
       </c>
-      <c r="O7" t="n">
+      <c r="S7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="P7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
+      <c r="T7" t="b">
+        <v>1</v>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="S7" t="n">
+      <c r="W7" t="n">
         <v>781</v>
       </c>
-      <c r="T7" t="n">
+      <c r="X7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="U7" t="b">
-        <v>1</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
+      <c r="Y7" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="n">
         <v>0.8962868117797695</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AC7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1093,63 +1220,80 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>[6, 1, 0, 6]</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="J8" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="K8" t="b">
+        <v>1</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>[6, 0, 6]</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="M8" t="n">
         <v>1419</v>
       </c>
-      <c r="J8" t="n">
+      <c r="N8" t="n">
         <v>55.44764714720212</v>
       </c>
-      <c r="K8" t="b">
-        <v>1</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
+      <c r="O8" t="b">
+        <v>1</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
         <is>
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="N8" t="n">
+      <c r="R8" t="n">
         <v>2075</v>
       </c>
-      <c r="O8" t="n">
+      <c r="S8" t="n">
         <v>77.62623579449122</v>
       </c>
-      <c r="P8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
+      <c r="T8" t="b">
+        <v>1</v>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
         <is>
           <t>[6, 1, 0, 6]</t>
         </is>
       </c>
-      <c r="S8" t="n">
+      <c r="W8" t="n">
         <v>2021</v>
       </c>
-      <c r="T8" t="n">
+      <c r="X8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="U8" t="b">
-        <v>1</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" t="n">
+      <c r="Y8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB8" t="n">
         <v>29.78723404255319</v>
       </c>
-      <c r="X8" t="n">
+      <c r="AC8" t="n">
         <v>-2.671944581890153</v>
       </c>
     </row>
@@ -1179,64 +1323,81 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>[7, 8, 7]</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>2291</v>
+      </c>
+      <c r="J9" t="n">
+        <v>72.81063071208843</v>
+      </c>
+      <c r="K9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="M9" t="n">
         <v>1379</v>
       </c>
-      <c r="J9" t="n">
+      <c r="N9" t="n">
         <v>76.21384847316919</v>
       </c>
-      <c r="K9" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M9" t="inlineStr">
+      <c r="O9" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
         <is>
           <t>[7, 8, 6, 7]</t>
         </is>
       </c>
-      <c r="N9" t="n">
+      <c r="R9" t="n">
         <v>55</v>
       </c>
-      <c r="O9" t="n">
+      <c r="S9" t="n">
         <v>76.21384847316919</v>
       </c>
-      <c r="P9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>[7, 6, 8, 7]</t>
-        </is>
-      </c>
-      <c r="S9" t="n">
-        <v>2169</v>
-      </c>
-      <c r="T9" t="n">
-        <v>76.25197526044872</v>
-      </c>
-      <c r="U9" t="b">
-        <v>1</v>
-      </c>
-      <c r="V9" t="n">
-        <v>-5.624711848778239</v>
+      <c r="T9" t="b">
+        <v>1</v>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>[7, 8, 7]</t>
+        </is>
       </c>
       <c r="W9" t="n">
-        <v>36.42231443061318</v>
+        <v>2291</v>
       </c>
       <c r="X9" t="n">
-        <v>97.46426924850161</v>
+        <v>72.81063071208843</v>
+      </c>
+      <c r="Y9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>39.80794412920122</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>97.59930161501528</v>
       </c>
     </row>
     <row r="10">
@@ -1265,63 +1426,80 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>[8, 2, 1, 8]</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>1707</v>
+      </c>
+      <c r="J10" t="n">
+        <v>70.15987690240341</v>
+      </c>
+      <c r="K10" t="b">
+        <v>1</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="M10" t="n">
         <v>1500</v>
       </c>
-      <c r="J10" t="n">
+      <c r="N10" t="n">
         <v>69.40771788690013</v>
       </c>
-      <c r="K10" t="b">
-        <v>1</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M10" t="inlineStr">
+      <c r="O10" t="b">
+        <v>1</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
         <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="N10" t="n">
+      <c r="R10" t="n">
         <v>1357</v>
       </c>
-      <c r="O10" t="n">
+      <c r="S10" t="n">
         <v>69.40771788690013</v>
       </c>
-      <c r="P10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
+      <c r="T10" t="b">
+        <v>1</v>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="S10" t="n">
+      <c r="W10" t="n">
         <v>1707</v>
       </c>
-      <c r="T10" t="n">
+      <c r="X10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="U10" t="b">
-        <v>1</v>
-      </c>
-      <c r="V10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W10" t="n">
+      <c r="Y10" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB10" t="n">
         <v>12.12653778558875</v>
       </c>
-      <c r="X10" t="n">
+      <c r="AC10" t="n">
         <v>20.50380785002929</v>
       </c>
     </row>
@@ -1365,49 +1543,66 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="M11" t="inlineStr">
-        <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
+      <c r="M11" t="n">
+        <v>-4042</v>
+      </c>
       <c r="N11" t="n">
+        <v>64.70237352474922</v>
+      </c>
+      <c r="O11" t="b">
+        <v>1</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>[9, 2, 9]</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
         <v>-4042</v>
       </c>
-      <c r="O11" t="n">
+      <c r="S11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="P11" t="b">
-        <v>1</v>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>Optimal</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
+      <c r="T11" t="b">
+        <v>1</v>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="S11" t="n">
+      <c r="W11" t="n">
         <v>-4042</v>
       </c>
-      <c r="T11" t="n">
+      <c r="X11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="U11" t="b">
-        <v>1</v>
-      </c>
-      <c r="V11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X11" t="n">
+      <c r="Y11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1438,7 +1633,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Oracle Avg Reward</t>
+          <t>MIP-Exact Avg Reward</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -1478,37 +1673,37 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Oracle Avg Inference (ms)</t>
+          <t>MIP-Exact Avg Inference (ms)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Avg Gap vs Oracle (%)</t>
+          <t>DRL Real Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Max Gap vs Oracle (%)</t>
+          <t>DRL Real Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Avg Gap vs Oracle (%)</t>
+          <t>HGA-LNS Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Max Gap vs Oracle (%)</t>
+          <t>HGA-LNS Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Avg Gap vs Oracle (%)</t>
+          <t>RH-Greedy Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Max Gap vs Oracle (%)</t>
+          <t>RH-Greedy Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1717,7 @@
         <v>10</v>
       </c>
       <c r="C2" t="n">
-        <v>1031.2</v>
+        <v>1156.6</v>
       </c>
       <c r="D2" t="n">
         <v>1059.9</v>
@@ -1534,37 +1729,37 @@
         <v>538.9</v>
       </c>
       <c r="G2" t="n">
-        <v>1122.513127326965</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>31.96866512298584</v>
+        <v>64.85259532928467</v>
       </c>
       <c r="I2" t="n">
-        <v>336.9940280914307</v>
+        <v>336.1144781112671</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8633852005004883</v>
+        <v>0.7659435272216797</v>
       </c>
       <c r="K2" t="n">
-        <v>96.12500667572021</v>
+        <v>223.1638669967651</v>
       </c>
       <c r="L2" t="n">
-        <v>-1.755522450761485</v>
+        <v>3.889782783588093</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>38.89782783588093</v>
       </c>
       <c r="N2" t="n">
-        <v>14.19563211736019</v>
+        <v>17.51308043057642</v>
       </c>
       <c r="O2" t="n">
-        <v>97.46426924850161</v>
+        <v>97.59930161501528</v>
       </c>
       <c r="P2" t="n">
-        <v>31.74815383217783</v>
+        <v>28.11102110179214</v>
       </c>
       <c r="Q2" t="n">
-        <v>189.385065885798</v>
+        <v>149.1150442477876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Segunda evaluación tras reemplazo de Solvers
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -1729,19 +1729,19 @@
         <v>538.9</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1280.436048984528</v>
       </c>
       <c r="H2" t="n">
-        <v>64.85259532928467</v>
+        <v>29.60474491119385</v>
       </c>
       <c r="I2" t="n">
-        <v>336.1144781112671</v>
+        <v>338.9090538024902</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7659435272216797</v>
+        <v>0.7550239562988281</v>
       </c>
       <c r="K2" t="n">
-        <v>223.1638669967651</v>
+        <v>220.9776878356934</v>
       </c>
       <c r="L2" t="n">
         <v>3.889782783588093</v>

</xml_diff>

<commit_message>
Tercera evaluación tras reemplazo de Solvers
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -620,7 +620,7 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>2054</v>
+        <v>2041</v>
       </c>
       <c r="N2" t="n">
         <v>76.7052345103569</v>
@@ -635,14 +635,14 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>[0, 1, 6, 0]</t>
+          <t>[0, 6, 0]</t>
         </is>
       </c>
       <c r="R2" t="n">
-        <v>1727</v>
+        <v>1459</v>
       </c>
       <c r="S2" t="n">
-        <v>77.62623579449122</v>
+        <v>55.44764714720212</v>
       </c>
       <c r="T2" t="b">
         <v>1</v>
@@ -673,10 +673,10 @@
         <v>0</v>
       </c>
       <c r="AB2" t="n">
-        <v>-0.6369426751592357</v>
+        <v>0</v>
       </c>
       <c r="AC2" t="n">
-        <v>15.38461538461539</v>
+        <v>28.51543361097501</v>
       </c>
     </row>
     <row r="3">
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>1164</v>
+        <v>1455</v>
       </c>
       <c r="N3" t="n">
         <v>69.40771788690012</v>
@@ -738,14 +738,14 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>[1, 6, 0, 1]</t>
+          <t>[1, 2, 8, 1]</t>
         </is>
       </c>
       <c r="R3" t="n">
-        <v>1928</v>
+        <v>1455</v>
       </c>
       <c r="S3" t="n">
-        <v>77.62623579449122</v>
+        <v>69.40771788690012</v>
       </c>
       <c r="T3" t="b">
         <v>1</v>
@@ -776,10 +776,10 @@
         <v>0</v>
       </c>
       <c r="AB3" t="n">
-        <v>29.71014492753623</v>
+        <v>12.13768115942029</v>
       </c>
       <c r="AC3" t="n">
-        <v>-16.42512077294686</v>
+        <v>12.13768115942029</v>
       </c>
     </row>
     <row r="4">
@@ -826,7 +826,7 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>-1221</v>
+        <v>2486</v>
       </c>
       <c r="N4" t="n">
         <v>72.44731374037281</v>
@@ -841,14 +841,14 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>[2, 8, 6, 2]</t>
+          <t>[2, 6, 8, 2]</t>
         </is>
       </c>
       <c r="R4" t="n">
-        <v>976</v>
+        <v>2486</v>
       </c>
       <c r="S4" t="n">
-        <v>72.45471862628276</v>
+        <v>72.44731374037281</v>
       </c>
       <c r="T4" t="b">
         <v>1</v>
@@ -879,10 +879,10 @@
         <v>38.89782783588093</v>
       </c>
       <c r="AB4" t="n">
-        <v>149.1150442477876</v>
+        <v>0</v>
       </c>
       <c r="AC4" t="n">
-        <v>60.74014481094127</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>1282</v>
+        <v>1344</v>
       </c>
       <c r="N5" t="n">
         <v>40.68356024804761</v>
@@ -982,7 +982,7 @@
         <v>0</v>
       </c>
       <c r="AB5" t="n">
-        <v>4.613095238095238</v>
+        <v>0</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>1080</v>
+        <v>1281</v>
       </c>
       <c r="N6" t="n">
         <v>40.68356024804761</v>
@@ -1085,7 +1085,7 @@
         <v>0</v>
       </c>
       <c r="AB6" t="n">
-        <v>15.69086651053864</v>
+        <v>0</v>
       </c>
       <c r="AC6" t="n">
         <v>0</v>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>774</v>
+        <v>781</v>
       </c>
       <c r="N7" t="n">
         <v>48.69171070169158</v>
@@ -1188,7 +1188,7 @@
         <v>0</v>
       </c>
       <c r="AB7" t="n">
-        <v>0.8962868117797695</v>
+        <v>0</v>
       </c>
       <c r="AC7" t="n">
         <v>0</v>
@@ -1238,7 +1238,7 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>1419</v>
+        <v>1828</v>
       </c>
       <c r="N8" t="n">
         <v>55.44764714720212</v>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Optimal</t>
+          <t>Infeasible</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1256,14 +1256,18 @@
           <t>[6, 0, 1, 6]</t>
         </is>
       </c>
-      <c r="R8" t="n">
-        <v>2075</v>
-      </c>
-      <c r="S8" t="n">
-        <v>77.62623579449122</v>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
       </c>
       <c r="T8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U8" t="inlineStr">
         <is>
@@ -1291,11 +1295,9 @@
         <v>0</v>
       </c>
       <c r="AB8" t="n">
-        <v>29.78723404255319</v>
-      </c>
-      <c r="AC8" t="n">
-        <v>-2.671944581890153</v>
-      </c>
+        <v>9.549727857496288</v>
+      </c>
+      <c r="AC8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1341,7 +1343,7 @@
         </is>
       </c>
       <c r="M9" t="n">
-        <v>1379</v>
+        <v>55</v>
       </c>
       <c r="N9" t="n">
         <v>76.21384847316919</v>
@@ -1356,14 +1358,14 @@
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>[7, 8, 6, 7]</t>
+          <t>[7, 6, 8, 7]</t>
         </is>
       </c>
       <c r="R9" t="n">
-        <v>55</v>
+        <v>2169</v>
       </c>
       <c r="S9" t="n">
-        <v>76.21384847316919</v>
+        <v>76.25197526044872</v>
       </c>
       <c r="T9" t="b">
         <v>1</v>
@@ -1394,10 +1396,10 @@
         <v>0</v>
       </c>
       <c r="AB9" t="n">
-        <v>39.80794412920122</v>
+        <v>97.59930161501528</v>
       </c>
       <c r="AC9" t="n">
-        <v>97.59930161501528</v>
+        <v>5.325185508511567</v>
       </c>
     </row>
     <row r="10">
@@ -1444,7 +1446,7 @@
         </is>
       </c>
       <c r="M10" t="n">
-        <v>1500</v>
+        <v>1357</v>
       </c>
       <c r="N10" t="n">
         <v>69.40771788690013</v>
@@ -1459,14 +1461,14 @@
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>[8, 1, 2, 8]</t>
+          <t>[8, 2, 1, 8]</t>
         </is>
       </c>
       <c r="R10" t="n">
-        <v>1357</v>
+        <v>1707</v>
       </c>
       <c r="S10" t="n">
-        <v>69.40771788690013</v>
+        <v>70.15987690240341</v>
       </c>
       <c r="T10" t="b">
         <v>1</v>
@@ -1497,10 +1499,10 @@
         <v>0</v>
       </c>
       <c r="AB10" t="n">
-        <v>12.12653778558875</v>
+        <v>20.50380785002929</v>
       </c>
       <c r="AC10" t="n">
-        <v>20.50380785002929</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -1723,25 +1725,25 @@
         <v>1059.9</v>
       </c>
       <c r="E2" t="n">
-        <v>748.2</v>
+        <v>960</v>
       </c>
       <c r="F2" t="n">
-        <v>538.9</v>
+        <v>858.6</v>
       </c>
       <c r="G2" t="n">
-        <v>1280.436048984528</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>29.60474491119385</v>
+        <v>64.1481876373291</v>
       </c>
       <c r="I2" t="n">
-        <v>338.9090538024902</v>
+        <v>233.1301689147949</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7550239562988281</v>
+        <v>1.010823249816895</v>
       </c>
       <c r="K2" t="n">
-        <v>220.9776878356934</v>
+        <v>216.1799669265747</v>
       </c>
       <c r="L2" t="n">
         <v>3.889782783588093</v>
@@ -1750,16 +1752,16 @@
         <v>38.89782783588093</v>
       </c>
       <c r="N2" t="n">
-        <v>17.51308043057642</v>
+        <v>5.108700030989652</v>
       </c>
       <c r="O2" t="n">
+        <v>28.51543361097501</v>
+      </c>
+      <c r="P2" t="n">
+        <v>13.97905184819612</v>
+      </c>
+      <c r="Q2" t="n">
         <v>97.59930161501528</v>
-      </c>
-      <c r="P2" t="n">
-        <v>28.11102110179214</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>149.1150442477876</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Evaluación estable tras reemplazo de Solvers
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -1251,11 +1251,7 @@
           <t>Infeasible</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>[6, 0, 1, 6]</t>
-        </is>
-      </c>
+      <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr">
         <is>
           <t>-inf</t>
@@ -1734,16 +1730,16 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>64.1481876373291</v>
+        <v>65.80398082733154</v>
       </c>
       <c r="I2" t="n">
-        <v>233.1301689147949</v>
+        <v>242.1642541885376</v>
       </c>
       <c r="J2" t="n">
-        <v>1.010823249816895</v>
+        <v>0.9992122650146484</v>
       </c>
       <c r="K2" t="n">
-        <v>216.1799669265747</v>
+        <v>220.9354162216187</v>
       </c>
       <c r="L2" t="n">
         <v>3.889782783588093</v>

</xml_diff>

<commit_message>
Primeros resultados al añadir Greedy RH estocastico
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC11"/>
+  <dimension ref="A1:AG11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,70 +507,90 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>RH-Greedy Real Route</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Greedy Real Reward</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Greedy Real Duration</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Greedy Real Valid</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>HGA-LNS Status</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Route</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Reward</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Duration</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Valid</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Status</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Route</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Reward</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Duration</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Valid</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs DRL Det (%)</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs DRL Real (%)</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs RH-Greedy (%)</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs HGA-LNS (%)</t>
         </is>
@@ -630,52 +650,66 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>[0, 6, 1, 0]</t>
+        </is>
+      </c>
+      <c r="Q2" t="n">
+        <v>2041</v>
+      </c>
+      <c r="R2" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="S2" t="b">
+        <v>1</v>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>[0, 6, 0]</t>
         </is>
       </c>
-      <c r="R2" t="n">
+      <c r="V2" t="n">
         <v>1459</v>
       </c>
-      <c r="S2" t="n">
+      <c r="W2" t="n">
         <v>55.44764714720212</v>
       </c>
-      <c r="T2" t="b">
-        <v>1</v>
-      </c>
-      <c r="U2" t="inlineStr">
+      <c r="X2" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y2" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>[0, 6, 1, 0]</t>
         </is>
       </c>
-      <c r="W2" t="n">
+      <c r="AA2" t="n">
         <v>2041</v>
       </c>
-      <c r="X2" t="n">
+      <c r="AB2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="Y2" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC2" t="n">
+      <c r="AC2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG2" t="n">
         <v>28.51543361097501</v>
       </c>
     </row>
@@ -733,52 +767,66 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>[1, 2, 8, 1]</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>1455</v>
+      </c>
+      <c r="R3" t="n">
+        <v>69.40771788690012</v>
+      </c>
+      <c r="S3" t="b">
+        <v>1</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>[1, 2, 8, 1]</t>
         </is>
       </c>
-      <c r="R3" t="n">
+      <c r="V3" t="n">
         <v>1455</v>
       </c>
-      <c r="S3" t="n">
+      <c r="W3" t="n">
         <v>69.40771788690012</v>
       </c>
-      <c r="T3" t="b">
-        <v>1</v>
-      </c>
-      <c r="U3" t="inlineStr">
+      <c r="X3" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>[1, 6, 8, 1]</t>
         </is>
       </c>
-      <c r="W3" t="n">
+      <c r="AA3" t="n">
         <v>1656</v>
       </c>
-      <c r="X3" t="n">
+      <c r="AB3" t="n">
         <v>76.66491525851202</v>
       </c>
-      <c r="Y3" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB3" t="n">
+      <c r="AC3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF3" t="n">
         <v>12.13768115942029</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AG3" t="n">
         <v>12.13768115942029</v>
       </c>
     </row>
@@ -836,52 +884,66 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
+          <t>[2, 6, 2]</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>1519</v>
+      </c>
+      <c r="R4" t="n">
+        <v>72.36542765017174</v>
+      </c>
+      <c r="S4" t="b">
+        <v>1</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="R4" t="n">
+      <c r="V4" t="n">
         <v>2486</v>
       </c>
-      <c r="S4" t="n">
+      <c r="W4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="T4" t="b">
-        <v>1</v>
-      </c>
-      <c r="U4" t="inlineStr">
+      <c r="X4" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="W4" t="n">
+      <c r="AA4" t="n">
         <v>2486</v>
       </c>
-      <c r="X4" t="n">
+      <c r="AB4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="Y4" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA4" t="n">
+      <c r="AC4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" t="n">
         <v>38.89782783588093</v>
       </c>
-      <c r="AB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC4" t="n">
+      <c r="AF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -939,52 +1001,66 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
+          <t>[3, 4, 3]</t>
+        </is>
+      </c>
+      <c r="Q5" t="n">
+        <v>1344</v>
+      </c>
+      <c r="R5" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="S5" t="b">
+        <v>1</v>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="R5" t="n">
+      <c r="V5" t="n">
         <v>1344</v>
       </c>
-      <c r="S5" t="n">
+      <c r="W5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="T5" t="b">
-        <v>1</v>
-      </c>
-      <c r="U5" t="inlineStr">
+      <c r="X5" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y5" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="W5" t="n">
+      <c r="AA5" t="n">
         <v>1344</v>
       </c>
-      <c r="X5" t="n">
+      <c r="AB5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="Y5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC5" t="n">
+      <c r="AC5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1042,52 +1118,66 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
+          <t>[4, 3, 4]</t>
+        </is>
+      </c>
+      <c r="Q6" t="n">
+        <v>1281</v>
+      </c>
+      <c r="R6" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="S6" t="b">
+        <v>1</v>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="R6" t="n">
+      <c r="V6" t="n">
         <v>1281</v>
       </c>
-      <c r="S6" t="n">
+      <c r="W6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="T6" t="b">
-        <v>1</v>
-      </c>
-      <c r="U6" t="inlineStr">
+      <c r="X6" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y6" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="W6" t="n">
+      <c r="AA6" t="n">
         <v>1281</v>
       </c>
-      <c r="X6" t="n">
+      <c r="AB6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="Y6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC6" t="n">
+      <c r="AC6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1145,52 +1235,66 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
+          <t>[5, 3, 5]</t>
+        </is>
+      </c>
+      <c r="Q7" t="n">
+        <v>781</v>
+      </c>
+      <c r="R7" t="n">
+        <v>48.69171070169158</v>
+      </c>
+      <c r="S7" t="b">
+        <v>1</v>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="R7" t="n">
+      <c r="V7" t="n">
         <v>781</v>
       </c>
-      <c r="S7" t="n">
+      <c r="W7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="T7" t="b">
-        <v>1</v>
-      </c>
-      <c r="U7" t="inlineStr">
+      <c r="X7" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y7" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="W7" t="n">
+      <c r="AA7" t="n">
         <v>781</v>
       </c>
-      <c r="X7" t="n">
+      <c r="AB7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="Y7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC7" t="n">
+      <c r="AC7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1248,52 +1352,66 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>[6, 0, 6]</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1828</v>
+      </c>
+      <c r="R8" t="n">
+        <v>55.44764714720212</v>
+      </c>
+      <c r="S8" t="b">
+        <v>1</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
           <t>Infeasible</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr">
+      <c r="U8" t="inlineStr"/>
+      <c r="V8" t="inlineStr">
         <is>
           <t>-inf</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>inf</t>
         </is>
       </c>
-      <c r="T8" t="b">
-        <v>0</v>
-      </c>
-      <c r="U8" t="inlineStr">
+      <c r="X8" t="b">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>[6, 1, 0, 6]</t>
         </is>
       </c>
-      <c r="W8" t="n">
+      <c r="AA8" t="n">
         <v>2021</v>
       </c>
-      <c r="X8" t="n">
+      <c r="AB8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="Y8" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB8" t="n">
+      <c r="AC8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
         <v>9.549727857496288</v>
       </c>
-      <c r="AC8" t="inlineStr"/>
+      <c r="AG8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1349,52 +1467,66 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
+          <t>[7, 6, 8, 7]</t>
+        </is>
+      </c>
+      <c r="Q9" t="n">
+        <v>2169</v>
+      </c>
+      <c r="R9" t="n">
+        <v>76.25197526044872</v>
+      </c>
+      <c r="S9" t="b">
+        <v>1</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>[7, 6, 8, 7]</t>
         </is>
       </c>
-      <c r="R9" t="n">
+      <c r="V9" t="n">
         <v>2169</v>
       </c>
-      <c r="S9" t="n">
+      <c r="W9" t="n">
         <v>76.25197526044872</v>
       </c>
-      <c r="T9" t="b">
-        <v>1</v>
-      </c>
-      <c r="U9" t="inlineStr">
+      <c r="X9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y9" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>[7, 8, 7]</t>
         </is>
       </c>
-      <c r="W9" t="n">
+      <c r="AA9" t="n">
         <v>2291</v>
       </c>
-      <c r="X9" t="n">
+      <c r="AB9" t="n">
         <v>72.81063071208843</v>
       </c>
-      <c r="Y9" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB9" t="n">
+      <c r="AC9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="n">
         <v>97.59930161501528</v>
       </c>
-      <c r="AC9" t="n">
+      <c r="AG9" t="n">
         <v>5.325185508511567</v>
       </c>
     </row>
@@ -1452,52 +1584,66 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
+          <t>[8, 1, 2, 8]</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1357</v>
+      </c>
+      <c r="R10" t="n">
+        <v>69.40771788690013</v>
+      </c>
+      <c r="S10" t="b">
+        <v>1</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="R10" t="n">
+      <c r="V10" t="n">
         <v>1707</v>
       </c>
-      <c r="S10" t="n">
+      <c r="W10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="T10" t="b">
-        <v>1</v>
-      </c>
-      <c r="U10" t="inlineStr">
+      <c r="X10" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y10" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="W10" t="n">
+      <c r="AA10" t="n">
         <v>1707</v>
       </c>
-      <c r="X10" t="n">
+      <c r="AB10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="Y10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB10" t="n">
+      <c r="AC10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="n">
         <v>20.50380785002929</v>
       </c>
-      <c r="AC10" t="n">
+      <c r="AG10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1553,54 +1699,68 @@
       <c r="O11" t="b">
         <v>1</v>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>-inf</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>inf</t>
+        </is>
+      </c>
+      <c r="S11" t="b">
+        <v>0</v>
+      </c>
+      <c r="T11" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="R11" t="n">
+      <c r="V11" t="n">
         <v>-4042</v>
       </c>
-      <c r="S11" t="n">
+      <c r="W11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="T11" t="b">
-        <v>1</v>
-      </c>
-      <c r="U11" t="inlineStr">
+      <c r="X11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Y11" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="W11" t="n">
+      <c r="AA11" t="n">
         <v>-4042</v>
       </c>
-      <c r="X11" t="n">
+      <c r="AB11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="Y11" t="b">
-        <v>1</v>
-      </c>
-      <c r="Z11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AA11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AB11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AC11" t="n">
+      <c r="AC11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1615,7 +1775,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1651,55 +1811,75 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>RH-Greedy Real Avg Reward</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Avg Reward (intersección)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Greedy Real Avg Reward (intersección)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>DRL Training Time (s)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Max Gap vs MIP-Exact (%)</t>
         </is>
@@ -1727,36 +1907,48 @@
         <v>858.6</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1530.555555555556</v>
       </c>
       <c r="H2" t="n">
-        <v>65.80398082733154</v>
+        <v>1626.777777777778</v>
       </c>
       <c r="I2" t="n">
-        <v>242.1642541885376</v>
+        <v>1530.555555555556</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9992122650146484</v>
+        <v>6.198813373422567</v>
       </c>
       <c r="K2" t="n">
-        <v>220.9354162216187</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
+        <v>65.22233486175537</v>
+      </c>
+      <c r="M2" t="n">
+        <v>233.2392692565918</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.9775876998901367</v>
+      </c>
+      <c r="O2" t="n">
+        <v>226.9024133682251</v>
+      </c>
+      <c r="P2" t="n">
         <v>3.889782783588093</v>
       </c>
-      <c r="M2" t="n">
+      <c r="Q2" t="n">
         <v>38.89782783588093</v>
       </c>
-      <c r="N2" t="n">
+      <c r="R2" t="n">
         <v>5.108700030989652</v>
       </c>
-      <c r="O2" t="n">
+      <c r="S2" t="n">
         <v>28.51543361097501</v>
       </c>
-      <c r="P2" t="n">
+      <c r="T2" t="n">
         <v>13.97905184819612</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="U2" t="n">
         <v>97.59930161501528</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Resultados estables con RH Greedy estocastico y RH lookahead deterministico
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG11"/>
+  <dimension ref="A1:AL11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,90 +507,115 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
+          <t>RH-Lookahead Route</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Reward</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Duration</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Valid</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>RH-Greedy Real Route</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Real Reward</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Real Duration</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Real Valid</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Status</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Route</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Reward</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Duration</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Valid</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Status</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Route</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Reward</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Duration</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Valid</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs DRL Det (%)</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs DRL Real (%)</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs RH-Greedy (%)</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>MIP-Exact Gap vs RH-Lookahead (%)</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs HGA-LNS (%)</t>
         </is>
@@ -664,53 +689,70 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
+          <t>[0, 6, 1, 0]</t>
+        </is>
+      </c>
+      <c r="U2" t="n">
+        <v>2041</v>
+      </c>
+      <c r="V2" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="W2" t="b">
+        <v>1</v>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>[0, 6, 0]</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>1459</v>
-      </c>
-      <c r="W2" t="n">
-        <v>55.44764714720212</v>
-      </c>
-      <c r="X2" t="b">
-        <v>1</v>
-      </c>
       <c r="Y2" t="inlineStr">
         <is>
+          <t>[0, 6, 1, 0]</t>
+        </is>
+      </c>
+      <c r="Z2" t="n">
+        <v>2041</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AB2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC2" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>[0, 6, 1, 0]</t>
         </is>
       </c>
-      <c r="AA2" t="n">
+      <c r="AE2" t="n">
         <v>2041</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AF2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AC2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG2" t="n">
-        <v>28.51543361097501</v>
+      <c r="AG2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -767,67 +809,84 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>[1, 6, 8, 1]</t>
+        </is>
+      </c>
+      <c r="Q3" t="n">
+        <v>1656</v>
+      </c>
+      <c r="R3" t="n">
+        <v>76.66491525851202</v>
+      </c>
+      <c r="S3" t="b">
+        <v>1</v>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
           <t>[1, 2, 8, 1]</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="U3" t="n">
         <v>1455</v>
       </c>
-      <c r="R3" t="n">
+      <c r="V3" t="n">
         <v>69.40771788690012</v>
       </c>
-      <c r="S3" t="b">
-        <v>1</v>
-      </c>
-      <c r="T3" t="inlineStr">
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+      <c r="X3" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>[1, 2, 8, 1]</t>
-        </is>
-      </c>
-      <c r="V3" t="n">
-        <v>1455</v>
-      </c>
-      <c r="W3" t="n">
-        <v>69.40771788690012</v>
-      </c>
-      <c r="X3" t="b">
-        <v>1</v>
-      </c>
       <c r="Y3" t="inlineStr">
         <is>
+          <t>[1, 6, 8, 1]</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>1656</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>76.66491525851202</v>
+      </c>
+      <c r="AB3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AD3" t="inlineStr">
         <is>
           <t>[1, 6, 8, 1]</t>
         </is>
       </c>
-      <c r="AA3" t="n">
+      <c r="AE3" t="n">
         <v>1656</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AF3" t="n">
         <v>76.66491525851202</v>
       </c>
-      <c r="AC3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF3" t="n">
+      <c r="AG3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" t="n">
         <v>12.13768115942029</v>
       </c>
-      <c r="AG3" t="n">
-        <v>12.13768115942029</v>
+      <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -884,66 +943,83 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
+          <t>[2, 6, 8, 2]</t>
+        </is>
+      </c>
+      <c r="Q4" t="n">
+        <v>2486</v>
+      </c>
+      <c r="R4" t="n">
+        <v>72.44731374037281</v>
+      </c>
+      <c r="S4" t="b">
+        <v>1</v>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
           <t>[2, 6, 2]</t>
         </is>
       </c>
-      <c r="Q4" t="n">
+      <c r="U4" t="n">
         <v>1519</v>
       </c>
-      <c r="R4" t="n">
+      <c r="V4" t="n">
         <v>72.36542765017174</v>
       </c>
-      <c r="S4" t="b">
-        <v>1</v>
-      </c>
-      <c r="T4" t="inlineStr">
+      <c r="W4" t="b">
+        <v>1</v>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="V4" t="n">
+      <c r="Z4" t="n">
         <v>2486</v>
       </c>
-      <c r="W4" t="n">
+      <c r="AA4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="X4" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AB4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="AA4" t="n">
+      <c r="AE4" t="n">
         <v>2486</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AF4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AC4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE4" t="n">
+      <c r="AG4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI4" t="n">
         <v>38.89782783588093</v>
       </c>
-      <c r="AF4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG4" t="n">
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1015,52 +1091,69 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
+          <t>[3, 4, 3]</t>
+        </is>
+      </c>
+      <c r="U5" t="n">
+        <v>1344</v>
+      </c>
+      <c r="V5" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="V5" t="n">
+      <c r="Z5" t="n">
         <v>1344</v>
       </c>
-      <c r="W5" t="n">
+      <c r="AA5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="X5" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AB5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC5" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AD5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AA5" t="n">
+      <c r="AE5" t="n">
         <v>1344</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AF5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AC5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG5" t="n">
+      <c r="AG5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1132,52 +1225,69 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
+          <t>[4, 3, 4]</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
+        <v>1281</v>
+      </c>
+      <c r="V6" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="W6" t="b">
+        <v>1</v>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="V6" t="n">
+      <c r="Z6" t="n">
         <v>1281</v>
       </c>
-      <c r="W6" t="n">
+      <c r="AA6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="X6" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AB6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC6" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AD6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AA6" t="n">
+      <c r="AE6" t="n">
         <v>1281</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AF6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AC6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG6" t="n">
+      <c r="AG6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1249,52 +1359,69 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
+          <t>[5, 3, 5]</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
+        <v>781</v>
+      </c>
+      <c r="V7" t="n">
+        <v>48.69171070169158</v>
+      </c>
+      <c r="W7" t="b">
+        <v>1</v>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="V7" t="n">
+      <c r="Z7" t="n">
         <v>781</v>
       </c>
-      <c r="W7" t="n">
+      <c r="AA7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="X7" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AB7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC7" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AD7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AA7" t="n">
+      <c r="AE7" t="n">
         <v>781</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AF7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AC7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" t="n">
+      <c r="AG7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1352,66 +1479,85 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>[6, 1, 0, 6]</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="R8" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="S8" t="b">
+        <v>1</v>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
           <t>[6, 0, 6]</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="U8" t="n">
         <v>1828</v>
       </c>
-      <c r="R8" t="n">
+      <c r="V8" t="n">
         <v>55.44764714720212</v>
       </c>
-      <c r="S8" t="b">
-        <v>1</v>
-      </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>Infeasible</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr"/>
-      <c r="V8" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="W8" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
-      </c>
-      <c r="X8" t="b">
-        <v>0</v>
+      <c r="W8" t="b">
+        <v>1</v>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>Optimal</t>
+        </is>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
+          <t>[6, 1, 0, 6]</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AB8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="AD8" t="inlineStr">
         <is>
           <t>[6, 1, 0, 6]</t>
         </is>
       </c>
-      <c r="AA8" t="n">
+      <c r="AE8" t="n">
         <v>2021</v>
       </c>
-      <c r="AB8" t="n">
+      <c r="AF8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AC8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" t="n">
+      <c r="AG8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="n">
         <v>9.549727857496288</v>
       </c>
-      <c r="AG8" t="inlineStr"/>
+      <c r="AK8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1481,53 +1627,70 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
+          <t>[7, 8, 7]</t>
+        </is>
+      </c>
+      <c r="U9" t="n">
+        <v>2291</v>
+      </c>
+      <c r="V9" t="n">
+        <v>72.81063071208843</v>
+      </c>
+      <c r="W9" t="b">
+        <v>1</v>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
-        <is>
-          <t>[7, 6, 8, 7]</t>
-        </is>
-      </c>
-      <c r="V9" t="n">
-        <v>2169</v>
-      </c>
-      <c r="W9" t="n">
-        <v>76.25197526044872</v>
-      </c>
-      <c r="X9" t="b">
-        <v>1</v>
-      </c>
       <c r="Y9" t="inlineStr">
         <is>
+          <t>[7, 8, 7]</t>
+        </is>
+      </c>
+      <c r="Z9" t="n">
+        <v>2291</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>72.81063071208843</v>
+      </c>
+      <c r="AB9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
+      <c r="AD9" t="inlineStr">
         <is>
           <t>[7, 8, 7]</t>
         </is>
       </c>
-      <c r="AA9" t="n">
+      <c r="AE9" t="n">
         <v>2291</v>
       </c>
-      <c r="AB9" t="n">
+      <c r="AF9" t="n">
         <v>72.81063071208843</v>
       </c>
-      <c r="AC9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF9" t="n">
+      <c r="AG9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
         <v>97.59930161501528</v>
       </c>
-      <c r="AG9" t="n">
+      <c r="AK9" t="n">
         <v>5.325185508511567</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1584,66 +1747,83 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
+          <t>[8, 2, 1, 8]</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1707</v>
+      </c>
+      <c r="R10" t="n">
+        <v>70.15987690240341</v>
+      </c>
+      <c r="S10" t="b">
+        <v>1</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
           <t>[8, 1, 2, 8]</t>
         </is>
       </c>
-      <c r="Q10" t="n">
+      <c r="U10" t="n">
         <v>1357</v>
       </c>
-      <c r="R10" t="n">
+      <c r="V10" t="n">
         <v>69.40771788690013</v>
       </c>
-      <c r="S10" t="b">
-        <v>1</v>
-      </c>
-      <c r="T10" t="inlineStr">
+      <c r="W10" t="b">
+        <v>1</v>
+      </c>
+      <c r="X10" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="V10" t="n">
+      <c r="Z10" t="n">
         <v>1707</v>
       </c>
-      <c r="W10" t="n">
+      <c r="AA10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="X10" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y10" t="inlineStr">
+      <c r="AB10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC10" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="AD10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="AA10" t="n">
+      <c r="AE10" t="n">
         <v>1707</v>
       </c>
-      <c r="AB10" t="n">
+      <c r="AF10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="AC10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF10" t="n">
+      <c r="AG10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
         <v>20.50380785002929</v>
       </c>
-      <c r="AG10" t="n">
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1699,68 +1879,85 @@
       <c r="O11" t="b">
         <v>1</v>
       </c>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>-inf</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr">
-        <is>
-          <t>inf</t>
-        </is>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>[9, 2, 9]</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>-4042</v>
+      </c>
+      <c r="R11" t="n">
+        <v>64.70237352474922</v>
       </c>
       <c r="S11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T11" t="inlineStr">
         <is>
+          <t>[9, 2, 9]</t>
+        </is>
+      </c>
+      <c r="U11" t="n">
+        <v>-4042</v>
+      </c>
+      <c r="V11" t="n">
+        <v>64.70237352474922</v>
+      </c>
+      <c r="W11" t="b">
+        <v>1</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="V11" t="n">
+      <c r="Z11" t="n">
         <v>-4042</v>
       </c>
-      <c r="W11" t="n">
+      <c r="AA11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="X11" t="b">
-        <v>1</v>
-      </c>
-      <c r="Y11" t="inlineStr">
+      <c r="AB11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AC11" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr">
+      <c r="AD11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AA11" t="n">
+      <c r="AE11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AB11" t="n">
+      <c r="AF11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AC11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AD11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AE11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG11" t="n">
+      <c r="AG11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1775,7 +1972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1811,77 +2008,87 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>RH-Lookahead Avg Reward</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>RH-Greedy Real Avg Reward</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>DRL Real Avg Reward (intersección)</t>
-        </is>
-      </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Real Avg Reward (intersección)</t>
+          <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
+          <t>DRL Training Time (s)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>DRL Training Time (s)</t>
+          <t>DRL Real Avg Inference (ms)</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Avg Inference (ms)</t>
+          <t>HGA-LNS Avg Inference (ms)</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Avg Inference (ms)</t>
+          <t>RH-Greedy Avg Inference (ms)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Avg Inference (ms)</t>
+          <t>MIP-Exact Avg Inference (ms)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>MIP-Exact Avg Inference (ms)</t>
+          <t>DRL Real Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Avg Gap vs MIP-Exact (%)</t>
+          <t>DRL Real Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>DRL Real Max Gap vs MIP-Exact (%)</t>
+          <t>HGA-LNS Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Avg Gap vs MIP-Exact (%)</t>
+          <t>HGA-LNS Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>HGA-LNS Max Gap vs MIP-Exact (%)</t>
+          <t>RH-Greedy Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Avg Gap vs MIP-Exact (%)</t>
+          <t>RH-Greedy Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>RH-Greedy Max Gap vs MIP-Exact (%)</t>
+          <t>RH-Lookahead Avg Gap vs MIP-Exact (%)</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Max Gap vs MIP-Exact (%)</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Avg Inference (ms)</t>
         </is>
       </c>
     </row>
@@ -1901,55 +2108,61 @@
         <v>1059.9</v>
       </c>
       <c r="E2" t="n">
-        <v>960</v>
+        <v>1156.6</v>
       </c>
       <c r="F2" t="n">
         <v>858.6</v>
       </c>
       <c r="G2" t="n">
-        <v>1530.555555555556</v>
+        <v>1144.4</v>
       </c>
       <c r="H2" t="n">
-        <v>1626.777777777778</v>
+        <v>985.5</v>
       </c>
       <c r="I2" t="n">
-        <v>1530.555555555556</v>
+        <v>5.016460851202487</v>
       </c>
       <c r="J2" t="n">
-        <v>6.198813373422567</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>65.53668975830078</v>
       </c>
       <c r="L2" t="n">
-        <v>65.22233486175537</v>
+        <v>473.1603860855103</v>
       </c>
       <c r="M2" t="n">
-        <v>233.2392692565918</v>
+        <v>0.949549674987793</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9775876998901367</v>
+        <v>220.2479362487793</v>
       </c>
       <c r="O2" t="n">
-        <v>226.9024133682251</v>
+        <v>3.889782783588093</v>
       </c>
       <c r="P2" t="n">
-        <v>3.889782783588093</v>
+        <v>38.89782783588093</v>
       </c>
       <c r="Q2" t="n">
-        <v>38.89782783588093</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>5.108700030989652</v>
+        <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>28.51543361097501</v>
+        <v>13.97905184819612</v>
       </c>
       <c r="T2" t="n">
-        <v>13.97905184819612</v>
+        <v>97.59930161501528</v>
       </c>
       <c r="U2" t="n">
-        <v>97.59930161501528</v>
+        <v>0.5325185508511567</v>
+      </c>
+      <c r="V2" t="n">
+        <v>5.325185508511567</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0.9557723999023438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resultados estables con RH lookahead estoastico
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL11"/>
+  <dimension ref="A1:AP11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -547,75 +547,95 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
+          <t>RH-Lookahead Real Route</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Real Reward</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Real Duration</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Real Valid</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>HGA-LNS Status</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Route</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Reward</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Duration</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Valid</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Status</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Route</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Reward</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Duration</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Valid</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs DRL Det (%)</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs DRL Real (%)</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs RH-Greedy (%)</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs RH-Lookahead (%)</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs HGA-LNS (%)</t>
         </is>
@@ -703,55 +723,69 @@
       </c>
       <c r="X2" t="inlineStr">
         <is>
+          <t>[0, 6, 1, 0]</t>
+        </is>
+      </c>
+      <c r="Y2" t="n">
+        <v>2041</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AA2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB2" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>[0, 6, 1, 0]</t>
         </is>
       </c>
-      <c r="Z2" t="n">
+      <c r="AD2" t="n">
         <v>2041</v>
       </c>
-      <c r="AA2" t="n">
+      <c r="AE2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AB2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AF2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG2" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>[0, 6, 1, 0]</t>
         </is>
       </c>
-      <c r="AE2" t="n">
+      <c r="AI2" t="n">
         <v>2041</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AJ2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AG2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>0</v>
+      <c r="AK2" t="b">
+        <v>1</v>
       </c>
       <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -837,55 +871,69 @@
       </c>
       <c r="X3" t="inlineStr">
         <is>
+          <t>[1, 6, 8, 1]</t>
+        </is>
+      </c>
+      <c r="Y3" t="n">
+        <v>1656</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>76.66491525851202</v>
+      </c>
+      <c r="AA3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>[1, 6, 8, 1]</t>
         </is>
       </c>
-      <c r="Z3" t="n">
+      <c r="AD3" t="n">
         <v>1656</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AE3" t="n">
         <v>76.66491525851202</v>
       </c>
-      <c r="AB3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AF3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG3" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD3" t="inlineStr">
+      <c r="AH3" t="inlineStr">
         <is>
           <t>[1, 6, 8, 1]</t>
         </is>
       </c>
-      <c r="AE3" t="n">
+      <c r="AI3" t="n">
         <v>1656</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AJ3" t="n">
         <v>76.66491525851202</v>
       </c>
-      <c r="AG3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ3" t="n">
+      <c r="AK3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN3" t="n">
         <v>12.13768115942029</v>
       </c>
-      <c r="AK3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL3" t="n">
+      <c r="AO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -971,55 +1019,69 @@
       </c>
       <c r="X4" t="inlineStr">
         <is>
+          <t>[2, 6, 2]</t>
+        </is>
+      </c>
+      <c r="Y4" t="n">
+        <v>1519</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>72.36542765017174</v>
+      </c>
+      <c r="AA4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="Z4" t="n">
+      <c r="AD4" t="n">
         <v>2486</v>
       </c>
-      <c r="AA4" t="n">
+      <c r="AE4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AB4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AF4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG4" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="AE4" t="n">
+      <c r="AI4" t="n">
         <v>2486</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AJ4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AG4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI4" t="n">
+      <c r="AK4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM4" t="n">
         <v>38.89782783588093</v>
       </c>
-      <c r="AJ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL4" t="n">
+      <c r="AN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1105,55 +1167,69 @@
       </c>
       <c r="X5" t="inlineStr">
         <is>
+          <t>[3, 4, 3]</t>
+        </is>
+      </c>
+      <c r="Y5" t="n">
+        <v>1344</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="AA5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="Z5" t="n">
+      <c r="AD5" t="n">
         <v>1344</v>
       </c>
-      <c r="AA5" t="n">
+      <c r="AE5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AB5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AF5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG5" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD5" t="inlineStr">
+      <c r="AH5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AE5" t="n">
+      <c r="AI5" t="n">
         <v>1344</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AJ5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AG5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0</v>
+      <c r="AK5" t="b">
+        <v>1</v>
       </c>
       <c r="AL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1239,55 +1315,69 @@
       </c>
       <c r="X6" t="inlineStr">
         <is>
+          <t>[4, 3, 4]</t>
+        </is>
+      </c>
+      <c r="Y6" t="n">
+        <v>1281</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="AA6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="Z6" t="n">
+      <c r="AD6" t="n">
         <v>1281</v>
       </c>
-      <c r="AA6" t="n">
+      <c r="AE6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AB6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AF6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG6" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD6" t="inlineStr">
+      <c r="AH6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AE6" t="n">
+      <c r="AI6" t="n">
         <v>1281</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AJ6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AG6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>0</v>
+      <c r="AK6" t="b">
+        <v>1</v>
       </c>
       <c r="AL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1373,55 +1463,69 @@
       </c>
       <c r="X7" t="inlineStr">
         <is>
+          <t>[5, 3, 5]</t>
+        </is>
+      </c>
+      <c r="Y7" t="n">
+        <v>781</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>48.69171070169158</v>
+      </c>
+      <c r="AA7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="Z7" t="n">
+      <c r="AD7" t="n">
         <v>781</v>
       </c>
-      <c r="AA7" t="n">
+      <c r="AE7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AB7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AF7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG7" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD7" t="inlineStr">
+      <c r="AH7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AE7" t="n">
+      <c r="AI7" t="n">
         <v>781</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AJ7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AG7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0</v>
+      <c r="AK7" t="b">
+        <v>1</v>
       </c>
       <c r="AL7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1507,55 +1611,69 @@
       </c>
       <c r="X8" t="inlineStr">
         <is>
+          <t>[6, 1, 0, 6]</t>
+        </is>
+      </c>
+      <c r="Y8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AA8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>[6, 1, 0, 6]</t>
         </is>
       </c>
-      <c r="Z8" t="n">
+      <c r="AD8" t="n">
         <v>2021</v>
       </c>
-      <c r="AA8" t="n">
+      <c r="AE8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AB8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AF8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG8" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD8" t="inlineStr">
+      <c r="AH8" t="inlineStr">
         <is>
           <t>[6, 1, 0, 6]</t>
         </is>
       </c>
-      <c r="AE8" t="n">
+      <c r="AI8" t="n">
         <v>2021</v>
       </c>
-      <c r="AF8" t="n">
+      <c r="AJ8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AG8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ8" t="n">
+      <c r="AK8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN8" t="n">
         <v>9.549727857496288</v>
       </c>
-      <c r="AK8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL8" t="n">
+      <c r="AO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1641,55 +1759,69 @@
       </c>
       <c r="X9" t="inlineStr">
         <is>
+          <t>[7, 8, 7]</t>
+        </is>
+      </c>
+      <c r="Y9" t="n">
+        <v>2291</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>72.81063071208843</v>
+      </c>
+      <c r="AA9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="AC9" t="inlineStr">
         <is>
           <t>[7, 8, 7]</t>
         </is>
       </c>
-      <c r="Z9" t="n">
+      <c r="AD9" t="n">
         <v>2291</v>
       </c>
-      <c r="AA9" t="n">
+      <c r="AE9" t="n">
         <v>72.81063071208843</v>
       </c>
-      <c r="AB9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC9" t="inlineStr">
+      <c r="AF9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG9" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD9" t="inlineStr">
+      <c r="AH9" t="inlineStr">
         <is>
           <t>[7, 8, 7]</t>
         </is>
       </c>
-      <c r="AE9" t="n">
+      <c r="AI9" t="n">
         <v>2291</v>
       </c>
-      <c r="AF9" t="n">
+      <c r="AJ9" t="n">
         <v>72.81063071208843</v>
       </c>
-      <c r="AG9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ9" t="n">
+      <c r="AK9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" t="n">
         <v>97.59930161501528</v>
       </c>
-      <c r="AK9" t="n">
+      <c r="AO9" t="n">
         <v>5.325185508511567</v>
       </c>
-      <c r="AL9" t="n">
+      <c r="AP9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1775,55 +1907,69 @@
       </c>
       <c r="X10" t="inlineStr">
         <is>
+          <t>[8, 2, 1, 8]</t>
+        </is>
+      </c>
+      <c r="Y10" t="n">
+        <v>1707</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>70.15987690240341</v>
+      </c>
+      <c r="AA10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="Z10" t="n">
+      <c r="AD10" t="n">
         <v>1707</v>
       </c>
-      <c r="AA10" t="n">
+      <c r="AE10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="AB10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AF10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG10" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD10" t="inlineStr">
+      <c r="AH10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="AE10" t="n">
+      <c r="AI10" t="n">
         <v>1707</v>
       </c>
-      <c r="AF10" t="n">
+      <c r="AJ10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="AG10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ10" t="n">
+      <c r="AK10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN10" t="n">
         <v>20.50380785002929</v>
       </c>
-      <c r="AK10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL10" t="n">
+      <c r="AO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1909,55 +2055,69 @@
       </c>
       <c r="X11" t="inlineStr">
         <is>
+          <t>[9, 2, 9]</t>
+        </is>
+      </c>
+      <c r="Y11" t="n">
+        <v>-4042</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>64.70237352474922</v>
+      </c>
+      <c r="AA11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="Z11" t="n">
+      <c r="AD11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AA11" t="n">
+      <c r="AE11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AB11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AF11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AG11" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AD11" t="inlineStr">
+      <c r="AH11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AE11" t="n">
+      <c r="AI11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AF11" t="n">
+      <c r="AJ11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AG11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AH11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>0</v>
+      <c r="AK11" t="b">
+        <v>1</v>
       </c>
       <c r="AL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1972,7 +2132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2018,77 +2178,92 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>RH-Lookahead Real Avg Reward</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Advantage vs RH-Lookahead Real (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>DRL Training Time (s)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Avg Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Avg Inference (ms)</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Real Avg Inference (ms)</t>
         </is>
       </c>
     </row>
@@ -2120,49 +2295,58 @@
         <v>985.5</v>
       </c>
       <c r="I2" t="n">
+        <v>1059.9</v>
+      </c>
+      <c r="J2" t="n">
         <v>5.016460851202487</v>
       </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
       <c r="K2" t="n">
-        <v>65.53668975830078</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>473.1603860855103</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.949549674987793</v>
+        <v>64.57962989807129</v>
       </c>
       <c r="N2" t="n">
-        <v>220.2479362487793</v>
+        <v>488.0144357681274</v>
       </c>
       <c r="O2" t="n">
+        <v>0.9914636611938477</v>
+      </c>
+      <c r="P2" t="n">
+        <v>216.3535356521606</v>
+      </c>
+      <c r="Q2" t="n">
         <v>3.889782783588093</v>
       </c>
-      <c r="P2" t="n">
+      <c r="R2" t="n">
         <v>38.89782783588093</v>
       </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
       <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
         <v>13.97905184819612</v>
       </c>
-      <c r="T2" t="n">
+      <c r="V2" t="n">
         <v>97.59930161501528</v>
       </c>
-      <c r="U2" t="n">
+      <c r="W2" t="n">
         <v>0.5325185508511567</v>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>5.325185508511567</v>
       </c>
-      <c r="W2" t="n">
-        <v>0.9557723999023438</v>
+      <c r="Y2" t="n">
+        <v>0.9695768356323242</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>1.416444778442383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resultados estables con Monte Carlo Rollout estocastico
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AP11"/>
+  <dimension ref="A1:AU11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -567,77 +567,102 @@
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
+          <t>MC-Rollout Route</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>MC-Rollout Reward</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>MC-Rollout Duration</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>MC-Rollout Valid</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
           <t>HGA-LNS Status</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Route</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Reward</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Duration</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Valid</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Status</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Route</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Reward</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Duration</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Valid</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs DRL Det (%)</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs DRL Real (%)</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs RH-Greedy (%)</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs RH-Lookahead (%)</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>MIP-Exact Gap vs HGA-LNS (%)</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>MIP-Exact Gap vs MC-Rollout (%)</t>
         </is>
       </c>
     </row>
@@ -737,55 +762,72 @@
       </c>
       <c r="AB2" t="inlineStr">
         <is>
+          <t>[0, 6, 1, 0]</t>
+        </is>
+      </c>
+      <c r="AC2" t="n">
+        <v>2041</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AE2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF2" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AG2" t="inlineStr">
         <is>
           <t>[0, 6, 1, 0]</t>
         </is>
       </c>
-      <c r="AD2" t="n">
+      <c r="AH2" t="n">
         <v>2041</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AI2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AF2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AJ2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK2" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>[0, 6, 1, 0]</t>
         </is>
       </c>
-      <c r="AI2" t="n">
+      <c r="AM2" t="n">
         <v>2041</v>
       </c>
-      <c r="AJ2" t="n">
+      <c r="AN2" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AK2" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO2" t="n">
-        <v>0</v>
+      <c r="AO2" t="b">
+        <v>1</v>
       </c>
       <c r="AP2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -885,55 +927,72 @@
       </c>
       <c r="AB3" t="inlineStr">
         <is>
+          <t>[1, 6, 8, 1]</t>
+        </is>
+      </c>
+      <c r="AC3" t="n">
+        <v>1656</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>76.66491525851202</v>
+      </c>
+      <c r="AE3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AG3" t="inlineStr">
         <is>
           <t>[1, 6, 8, 1]</t>
         </is>
       </c>
-      <c r="AD3" t="n">
+      <c r="AH3" t="n">
         <v>1656</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AI3" t="n">
         <v>76.66491525851202</v>
       </c>
-      <c r="AF3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AJ3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK3" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AL3" t="inlineStr">
         <is>
           <t>[1, 6, 8, 1]</t>
         </is>
       </c>
-      <c r="AI3" t="n">
+      <c r="AM3" t="n">
         <v>1656</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AN3" t="n">
         <v>76.66491525851202</v>
       </c>
-      <c r="AK3" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN3" t="n">
+      <c r="AO3" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="n">
         <v>12.13768115942029</v>
       </c>
-      <c r="AO3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP3" t="n">
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1033,56 +1092,73 @@
       </c>
       <c r="AB4" t="inlineStr">
         <is>
+          <t>[2, 6, 2]</t>
+        </is>
+      </c>
+      <c r="AC4" t="n">
+        <v>1519</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>72.36542765017174</v>
+      </c>
+      <c r="AE4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AG4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="AD4" t="n">
+      <c r="AH4" t="n">
         <v>2486</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AI4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AF4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AJ4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK4" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>[2, 6, 8, 2]</t>
         </is>
       </c>
-      <c r="AI4" t="n">
+      <c r="AM4" t="n">
         <v>2486</v>
       </c>
-      <c r="AJ4" t="n">
+      <c r="AN4" t="n">
         <v>72.44731374037281</v>
       </c>
-      <c r="AK4" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM4" t="n">
+      <c r="AO4" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ4" t="n">
         <v>38.89782783588093</v>
       </c>
-      <c r="AN4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP4" t="n">
-        <v>0</v>
+      <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU4" t="n">
+        <v>38.89782783588093</v>
       </c>
     </row>
     <row r="5">
@@ -1181,55 +1257,72 @@
       </c>
       <c r="AB5" t="inlineStr">
         <is>
+          <t>[3, 4, 3]</t>
+        </is>
+      </c>
+      <c r="AC5" t="n">
+        <v>1344</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="AE5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AG5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AD5" t="n">
+      <c r="AH5" t="n">
         <v>1344</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AI5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AF5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG5" t="inlineStr">
+      <c r="AJ5" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK5" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AL5" t="inlineStr">
         <is>
           <t>[3, 4, 3]</t>
         </is>
       </c>
-      <c r="AI5" t="n">
+      <c r="AM5" t="n">
         <v>1344</v>
       </c>
-      <c r="AJ5" t="n">
+      <c r="AN5" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AK5" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO5" t="n">
-        <v>0</v>
+      <c r="AO5" t="b">
+        <v>1</v>
       </c>
       <c r="AP5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1329,55 +1422,72 @@
       </c>
       <c r="AB6" t="inlineStr">
         <is>
+          <t>[4, 3, 4]</t>
+        </is>
+      </c>
+      <c r="AC6" t="n">
+        <v>1281</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>40.68356024804761</v>
+      </c>
+      <c r="AE6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AG6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AD6" t="n">
+      <c r="AH6" t="n">
         <v>1281</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AI6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AF6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG6" t="inlineStr">
+      <c r="AJ6" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK6" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AL6" t="inlineStr">
         <is>
           <t>[4, 3, 4]</t>
         </is>
       </c>
-      <c r="AI6" t="n">
+      <c r="AM6" t="n">
         <v>1281</v>
       </c>
-      <c r="AJ6" t="n">
+      <c r="AN6" t="n">
         <v>40.68356024804761</v>
       </c>
-      <c r="AK6" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>0</v>
+      <c r="AO6" t="b">
+        <v>1</v>
       </c>
       <c r="AP6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1477,55 +1587,72 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
+          <t>[5, 3, 5]</t>
+        </is>
+      </c>
+      <c r="AC7" t="n">
+        <v>781</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>48.69171070169158</v>
+      </c>
+      <c r="AE7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AG7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AD7" t="n">
+      <c r="AH7" t="n">
         <v>781</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AI7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AF7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG7" t="inlineStr">
+      <c r="AJ7" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK7" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr">
+      <c r="AL7" t="inlineStr">
         <is>
           <t>[5, 3, 5]</t>
         </is>
       </c>
-      <c r="AI7" t="n">
+      <c r="AM7" t="n">
         <v>781</v>
       </c>
-      <c r="AJ7" t="n">
+      <c r="AN7" t="n">
         <v>48.69171070169158</v>
       </c>
-      <c r="AK7" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO7" t="n">
-        <v>0</v>
+      <c r="AO7" t="b">
+        <v>1</v>
       </c>
       <c r="AP7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1625,55 +1752,72 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
+          <t>[6, 1, 0, 6]</t>
+        </is>
+      </c>
+      <c r="AC8" t="n">
+        <v>2021</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>76.7052345103569</v>
+      </c>
+      <c r="AE8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC8" t="inlineStr">
+      <c r="AG8" t="inlineStr">
         <is>
           <t>[6, 1, 0, 6]</t>
         </is>
       </c>
-      <c r="AD8" t="n">
+      <c r="AH8" t="n">
         <v>2021</v>
       </c>
-      <c r="AE8" t="n">
+      <c r="AI8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AF8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG8" t="inlineStr">
+      <c r="AJ8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK8" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH8" t="inlineStr">
+      <c r="AL8" t="inlineStr">
         <is>
           <t>[6, 1, 0, 6]</t>
         </is>
       </c>
-      <c r="AI8" t="n">
+      <c r="AM8" t="n">
         <v>2021</v>
       </c>
-      <c r="AJ8" t="n">
+      <c r="AN8" t="n">
         <v>76.7052345103569</v>
       </c>
-      <c r="AK8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN8" t="n">
+      <c r="AO8" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" t="n">
         <v>9.549727857496288</v>
       </c>
-      <c r="AO8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP8" t="n">
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1773,55 +1917,72 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
+          <t>[7, 8, 7]</t>
+        </is>
+      </c>
+      <c r="AC9" t="n">
+        <v>2291</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>72.81063071208843</v>
+      </c>
+      <c r="AE9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC9" t="inlineStr">
+      <c r="AG9" t="inlineStr">
         <is>
           <t>[7, 8, 7]</t>
         </is>
       </c>
-      <c r="AD9" t="n">
+      <c r="AH9" t="n">
         <v>2291</v>
       </c>
-      <c r="AE9" t="n">
+      <c r="AI9" t="n">
         <v>72.81063071208843</v>
       </c>
-      <c r="AF9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG9" t="inlineStr">
+      <c r="AJ9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK9" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH9" t="inlineStr">
+      <c r="AL9" t="inlineStr">
         <is>
           <t>[7, 8, 7]</t>
         </is>
       </c>
-      <c r="AI9" t="n">
+      <c r="AM9" t="n">
         <v>2291</v>
       </c>
-      <c r="AJ9" t="n">
+      <c r="AN9" t="n">
         <v>72.81063071208843</v>
       </c>
-      <c r="AK9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN9" t="n">
+      <c r="AO9" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR9" t="n">
         <v>97.59930161501528</v>
       </c>
-      <c r="AO9" t="n">
+      <c r="AS9" t="n">
         <v>5.325185508511567</v>
       </c>
-      <c r="AP9" t="n">
+      <c r="AT9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1921,55 +2082,72 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
+          <t>[8, 2, 1, 8]</t>
+        </is>
+      </c>
+      <c r="AC10" t="n">
+        <v>1707</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>70.15987690240341</v>
+      </c>
+      <c r="AE10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC10" t="inlineStr">
+      <c r="AG10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="AD10" t="n">
+      <c r="AH10" t="n">
         <v>1707</v>
       </c>
-      <c r="AE10" t="n">
+      <c r="AI10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="AF10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG10" t="inlineStr">
+      <c r="AJ10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK10" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH10" t="inlineStr">
+      <c r="AL10" t="inlineStr">
         <is>
           <t>[8, 2, 1, 8]</t>
         </is>
       </c>
-      <c r="AI10" t="n">
+      <c r="AM10" t="n">
         <v>1707</v>
       </c>
-      <c r="AJ10" t="n">
+      <c r="AN10" t="n">
         <v>70.15987690240341</v>
       </c>
-      <c r="AK10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN10" t="n">
+      <c r="AO10" t="b">
+        <v>1</v>
+      </c>
+      <c r="AP10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR10" t="n">
         <v>20.50380785002929</v>
       </c>
-      <c r="AO10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP10" t="n">
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2069,55 +2247,72 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
+          <t>[9, 2, 9]</t>
+        </is>
+      </c>
+      <c r="AC11" t="n">
+        <v>-4042</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>64.70237352474922</v>
+      </c>
+      <c r="AE11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AC11" t="inlineStr">
+      <c r="AG11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AD11" t="n">
+      <c r="AH11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AE11" t="n">
+      <c r="AI11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AF11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG11" t="inlineStr">
+      <c r="AJ11" t="b">
+        <v>1</v>
+      </c>
+      <c r="AK11" t="inlineStr">
         <is>
           <t>Optimal</t>
         </is>
       </c>
-      <c r="AH11" t="inlineStr">
+      <c r="AL11" t="inlineStr">
         <is>
           <t>[9, 2, 9]</t>
         </is>
       </c>
-      <c r="AI11" t="n">
+      <c r="AM11" t="n">
         <v>-4042</v>
       </c>
-      <c r="AJ11" t="n">
+      <c r="AN11" t="n">
         <v>64.70237352474922</v>
       </c>
-      <c r="AK11" t="b">
-        <v>1</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO11" t="n">
-        <v>0</v>
+      <c r="AO11" t="b">
+        <v>1</v>
       </c>
       <c r="AP11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2132,7 +2327,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2266,6 +2461,31 @@
           <t>RH-Lookahead Real Avg Inference (ms)</t>
         </is>
       </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>MC-Rollout Avg Reward</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>MC-Rollout Avg Gap vs MIP-Exact (%)</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>MC-Rollout Max Gap vs MIP-Exact (%)</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>MC-Rollout Avg Inference (ms)</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Real Advantage vs MC-Rollout (%)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2307,16 +2527,16 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>64.57962989807129</v>
+        <v>65.04034996032715</v>
       </c>
       <c r="N2" t="n">
-        <v>488.0144357681274</v>
+        <v>478.1922578811646</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9914636611938477</v>
+        <v>0.9978294372558594</v>
       </c>
       <c r="P2" t="n">
-        <v>216.3535356521606</v>
+        <v>220.0825929641724</v>
       </c>
       <c r="Q2" t="n">
         <v>3.889782783588093</v>
@@ -2343,10 +2563,25 @@
         <v>5.325185508511567</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.9695768356323242</v>
+        <v>0.9304046630859375</v>
       </c>
       <c r="Z2" t="n">
-        <v>1.416444778442383</v>
+        <v>1.334762573242188</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>1059.9</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>3.889782783588093</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>38.89782783588093</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>29.26807403564453</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Nueva implementación MIP pero falla con 20 nodos
</commit_message>
<xml_diff>
--- a/results_10nodes/DRL_Routing_Summary_AM.xlsx
+++ b/results_10nodes/DRL_Routing_Summary_AM.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU11"/>
+  <dimension ref="A1:AO11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -612,57 +612,27 @@
       </c>
       <c r="AK1" s="1" t="inlineStr">
         <is>
-          <t>MIP-Exact Status</t>
+          <t>MIP Status</t>
         </is>
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>MIP-Exact Route</t>
+          <t>MIP Route</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
         <is>
-          <t>MIP-Exact Reward</t>
+          <t>MIP Reward</t>
         </is>
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>MIP-Exact Duration</t>
+          <t>MIP Duration</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
         <is>
-          <t>MIP-Exact Valid</t>
-        </is>
-      </c>
-      <c r="AP1" s="1" t="inlineStr">
-        <is>
-          <t>MIP-Exact Gap vs DRL Det (%)</t>
-        </is>
-      </c>
-      <c r="AQ1" s="1" t="inlineStr">
-        <is>
-          <t>MIP-Exact Gap vs DRL Real (%)</t>
-        </is>
-      </c>
-      <c r="AR1" s="1" t="inlineStr">
-        <is>
-          <t>MIP-Exact Gap vs RH-Greedy (%)</t>
-        </is>
-      </c>
-      <c r="AS1" s="1" t="inlineStr">
-        <is>
-          <t>MIP-Exact Gap vs RH-Lookahead (%)</t>
-        </is>
-      </c>
-      <c r="AT1" s="1" t="inlineStr">
-        <is>
-          <t>MIP-Exact Gap vs HGA-LNS (%)</t>
-        </is>
-      </c>
-      <c r="AU1" s="1" t="inlineStr">
-        <is>
-          <t>MIP-Exact Gap vs MC-Rollout (%)</t>
+          <t>MIP Valid</t>
         </is>
       </c>
     </row>
@@ -812,24 +782,6 @@
       <c r="AO2" t="b">
         <v>1</v>
       </c>
-      <c r="AP2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -976,24 +928,6 @@
       </c>
       <c r="AO3" t="b">
         <v>1</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR3" t="n">
-        <v>12.13768115942029</v>
-      </c>
-      <c r="AS3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU3" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -1142,24 +1076,6 @@
       <c r="AO4" t="b">
         <v>1</v>
       </c>
-      <c r="AP4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ4" t="n">
-        <v>38.89782783588093</v>
-      </c>
-      <c r="AR4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>38.89782783588093</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1307,24 +1223,6 @@
       <c r="AO5" t="b">
         <v>1</v>
       </c>
-      <c r="AP5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1472,24 +1370,6 @@
       <c r="AO6" t="b">
         <v>1</v>
       </c>
-      <c r="AP6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU6" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1637,24 +1517,6 @@
       <c r="AO7" t="b">
         <v>1</v>
       </c>
-      <c r="AP7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU7" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1802,24 +1664,6 @@
       <c r="AO8" t="b">
         <v>1</v>
       </c>
-      <c r="AP8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>9.549727857496288</v>
-      </c>
-      <c r="AS8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU8" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1967,24 +1811,6 @@
       <c r="AO9" t="b">
         <v>1</v>
       </c>
-      <c r="AP9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR9" t="n">
-        <v>97.59930161501528</v>
-      </c>
-      <c r="AS9" t="n">
-        <v>5.325185508511567</v>
-      </c>
-      <c r="AT9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU9" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -2132,24 +1958,6 @@
       <c r="AO10" t="b">
         <v>1</v>
       </c>
-      <c r="AP10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR10" t="n">
-        <v>20.50380785002929</v>
-      </c>
-      <c r="AS10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU10" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -2296,24 +2104,6 @@
       </c>
       <c r="AO11" t="b">
         <v>1</v>
-      </c>
-      <c r="AP11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU11" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2343,137 +2133,137 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>MIP-Exact Avg Reward</t>
+          <t>MIP Avg Reward</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>MIP Optimal Count</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>MIP Avg Inference (ms)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Avg Reward</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Gap vs MIP Avg (%)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>DRL Det Gap vs MIP Max (%)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>DRL Real Avg Reward</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Reward</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HGA-LNS Gap vs MIP Avg (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>HGA-LNS Gap vs MIP Max (%)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Reward</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Greedy Gap vs MIP Avg (%)</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Greedy Gap vs MIP Max (%)</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Avg Reward</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Gap vs MIP Avg (%)</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>RH-Lookahead Gap vs MIP Max (%)</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Real Avg Reward</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Real Avg Reward</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs RH-Greedy Real (%)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Advantage vs RH-Lookahead Real (%)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>DRL Training Time (s)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>DRL Real Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>HGA-LNS Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>RH-Greedy Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>MIP-Exact Avg Inference (ms)</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>DRL Real Avg Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>DRL Real Max Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>HGA-LNS Avg Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>HGA-LNS Max Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>RH-Greedy Avg Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>RH-Greedy Max Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>RH-Lookahead Avg Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>RH-Lookahead Max Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>RH-Lookahead Real Avg Inference (ms)</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>MC-Rollout Avg Reward</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>MC-Rollout Avg Gap vs MIP-Exact (%)</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>MC-Rollout Max Gap vs MIP-Exact (%)</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
@@ -2500,25 +2290,25 @@
         <v>1156.6</v>
       </c>
       <c r="D2" t="n">
-        <v>1059.9</v>
+        <v>10</v>
       </c>
       <c r="E2" t="n">
+        <v>4699.912142753601</v>
+      </c>
+      <c r="F2" t="n">
         <v>1156.6</v>
       </c>
-      <c r="F2" t="n">
-        <v>858.6</v>
-      </c>
       <c r="G2" t="n">
-        <v>1144.4</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>985.5</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
         <v>1059.9</v>
       </c>
       <c r="J2" t="n">
-        <v>5.016460851202487</v>
+        <v>1156.6</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
@@ -2527,58 +2317,58 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>65.04034996032715</v>
+        <v>858.6</v>
       </c>
       <c r="N2" t="n">
-        <v>478.1922578811646</v>
+        <v>13.97905184819612</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9978294372558594</v>
+        <v>97.59930161501528</v>
       </c>
       <c r="P2" t="n">
-        <v>220.0825929641724</v>
+        <v>1144.4</v>
       </c>
       <c r="Q2" t="n">
-        <v>3.889782783588093</v>
+        <v>0.5325185508511567</v>
       </c>
       <c r="R2" t="n">
-        <v>38.89782783588093</v>
+        <v>5.325185508511567</v>
       </c>
       <c r="S2" t="n">
+        <v>985.5</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1059.9</v>
+      </c>
+      <c r="U2" t="n">
+        <v>5.016460851202487</v>
+      </c>
+      <c r="V2" t="n">
         <v>0</v>
       </c>
-      <c r="T2" t="n">
+      <c r="W2" t="n">
         <v>0</v>
       </c>
-      <c r="U2" t="n">
-        <v>13.97905184819612</v>
-      </c>
-      <c r="V2" t="n">
-        <v>97.59930161501528</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0.5325185508511567</v>
-      </c>
       <c r="X2" t="n">
-        <v>5.325185508511567</v>
+        <v>177.039623260498</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.9304046630859375</v>
+        <v>479.9443244934082</v>
       </c>
       <c r="Z2" t="n">
-        <v>1.334762573242188</v>
+        <v>0.9086370468139648</v>
       </c>
       <c r="AA2" t="n">
+        <v>0.8826494216918945</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>1.280665397644043</v>
+      </c>
+      <c r="AC2" t="n">
         <v>1059.9</v>
       </c>
-      <c r="AB2" t="n">
-        <v>3.889782783588093</v>
-      </c>
-      <c r="AC2" t="n">
-        <v>38.89782783588093</v>
-      </c>
       <c r="AD2" t="n">
-        <v>29.26807403564453</v>
+        <v>29.73134517669678</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>

</xml_diff>